<commit_message>
Catálogo: importar la actualización del Excel (159 ítems)
26 ítems nuevos —13 armas y 13 escudos—, uno borrado y 15 con cambios de
precio, tier, peso o modificadores. Los escudos dejan de tener tipoDado,
que no les correspondía, y el bloqueo pasa a ser un modificador de
verdad en vez de texto suelto en el detalle.

Se completan los tipos que venían vacíos: 12 armas como arma_1m y 13
escudos como escudo_1m, siguiendo la regla de que por ahora todo es de
una mano. El Escudo romano pasa de dos manos a una, como quedó en el
Excel.

Esto además destraba el Vendor Generator: ahora hay 13 ítems
Excepcionales y 4 Legendarios, así que una Capital da 12,5% y 2,3%
contra el 15% y 3% de la tabla. Antes daba 3,1% y 0% porque no existían.

El Excel queda sincronizado con los IDs nuevos ya puestos, verificado
leyéndolo de vuelta: 159 de 159 sin diferencias.
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -16,8 +16,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Consumibles'!$A$1:$S$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$R$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Escudos'!$A$1:$R$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$R$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Escudos'!$A$1:$R$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defensivos'!$A$1:$AE$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Otros'!$A$1:$Q$2</definedName>
   </definedNames>
@@ -2069,7 +2069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2187,12 +2187,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>new-daga</t>
+          <t>new-daga-de-capitan</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Daga</t>
+          <t>Daga de Capitán</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2212,20 +2212,22 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Ignora 1 de resistencia crítica.</t>
+          <t>pdg +1</t>
         </is>
       </c>
       <c r="I2" t="n">
         <v>2</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -2237,12 +2239,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cat-espada-ancha</t>
+          <t>new-daga-de-guardia</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Espada ancha</t>
+          <t>Daga de guardia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2256,21 +2258,21 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>60</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Daño amplificado.</t>
+          <t>Ignora 1 punto de resistencia al crítico</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -2282,21 +2284,17 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cat-espada-larga</t>
+          <t>cat-espada-ancha</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Espada larga</t>
+          <t>Espada ancha</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2316,22 +2314,20 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Pdg +1</t>
+          <t>Daño amplificado.</t>
         </is>
       </c>
       <c r="I4" t="n">
         <v>4</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -2347,12 +2343,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cat-estoque</t>
+          <t>cat-espada-larga</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Estoque</t>
+          <t>Espada larga</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2372,24 +2368,24 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Modificador: '+1 a iniciativa</t>
+          <t>Pdg +1</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
@@ -2403,12 +2399,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cat-hacha-de-batalla</t>
+          <t>new-estilete-de-competencia</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hacha de batalla</t>
+          <t>Estilete de competencia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2425,18 +2421,18 @@
         <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Rompe armadura. +1 al bloqueo</t>
+          <t>Crítico +1</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -2446,25 +2442,19 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="n">
-        <v>1</v>
-      </c>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>new-hacha-de-guerra-ligera</t>
+          <t>cat-estoque</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hacha de guerra ligera</t>
+          <t>Estoque</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2478,43 +2468,49 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Rompe armadura</t>
+          <t>Modificador: +1 a iniciativa</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cat-martillo</t>
+          <t>cat-hacha-de-batalla</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Martillo</t>
+          <t>Hacha de batalla</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2528,31 +2524,33 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Daño +50%. Lento.</t>
+          <t>Rompe armadura. +1 al bloqueo</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="P8" t="n">
+        <v>1</v>
+      </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
@@ -2563,12 +2561,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>new-martillo-de-sargento</t>
+          <t>new-hacha-de-guerra-ligera</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Martillo de sargento</t>
+          <t>Hacha de guerra ligera</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2582,33 +2580,29 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Tipo de daño: Tipo 8 (Impacto/contundente).</t>
+          <t>Rompe armadura</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="n">
-        <v>10</v>
-      </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
@@ -2617,12 +2611,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cat-rompemalla</t>
+          <t>cat-martillo</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Rompemalla</t>
+          <t>Martillo</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2636,24 +2630,24 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>40</v>
+        <v>124</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Rompe armadura.</t>
+          <t>Daño +50%. Lento.</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
@@ -2671,12 +2665,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>new-sable-de-caballeria</t>
+          <t>new-martillo-de-sargento</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sable de caballería</t>
+          <t>Martillo de sargento</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2690,27 +2684,33 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>87</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
+        <v>112</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Tipo de daño: Tipo 8 (Impacto/contundente).</t>
+        </is>
+      </c>
       <c r="I11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>10</v>
+      </c>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
@@ -2719,17 +2719,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>new-cachiporra</t>
+          <t>new-pico-de-guerra</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cachiporra</t>
+          <t>Pico de guerra</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2738,29 +2738,27 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Tipo de daño: Tipo 8 (Impacto/contundente).</t>
+          <t>rango +1, 50% de romper armadura</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="n">
-        <v>10</v>
-      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
@@ -2771,17 +2769,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>new-cuchillo-de-cazador</t>
+          <t>cat-rompemalla</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cuchillo de cazador</t>
+          <t>Rompemalla</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2790,20 +2788,24 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>30</v>
-      </c>
-      <c r="H13" t="inlineStr"/>
+        <v>75</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>50% chance de Romper armadura.</t>
+        </is>
+      </c>
       <c r="I13" t="n">
         <v>2</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -2812,22 +2814,26 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cat-espada-corta</t>
+          <t>new-sable-de-caballeria</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Espada corta</t>
+          <t>Sable de caballería</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2836,43 +2842,41 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>new-espada-corta-de-instruccion</t>
+          <t>new-cachiporra</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Espada corta de instrucción</t>
+          <t>Cachiporra</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2886,17 +2890,21 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>50</v>
-      </c>
-      <c r="H15" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Tipo de daño: Tipo 8 (Impacto/contundente).</t>
+        </is>
+      </c>
       <c r="I15" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -2915,12 +2923,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cat-hacha</t>
+          <t>new-cuchillo-de-cazador</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Hacha</t>
+          <t>Cuchillo de cazador</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2940,15 +2948,11 @@
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>60</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Rompe armadura.</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -2960,21 +2964,17 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cat-machete</t>
+          <t>new-daga</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Machete</t>
+          <t>Daga</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2991,21 +2991,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>55</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>+10% de daño crítico</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -3014,21 +3010,17 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cat-maza</t>
+          <t>cat-espada-corta</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Maza</t>
+          <t>Espada corta</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3042,24 +3034,20 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>66</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Bloqueo +1</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -3077,12 +3065,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>new-maza-de-guardia</t>
+          <t>new-espada-corta-de-instruccion</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Maza de guardia</t>
+          <t>Espada corta de instrucción</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3096,27 +3084,25 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>55</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Bloqueo +1</t>
-        </is>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>10</v>
+      </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
@@ -3127,12 +3113,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>new-punal-de-asalto</t>
+          <t>new-estileto-comun</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Puñal de asalto</t>
+          <t>Estileto común</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3149,12 +3135,16 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>45</v>
-      </c>
-      <c r="H20" t="inlineStr"/>
+        <v>50</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>crítico +1</t>
+        </is>
+      </c>
       <c r="I20" t="n">
         <v>2</v>
       </c>
@@ -3173,17 +3163,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>new-espadon</t>
+          <t>cat-hacha</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Espadón</t>
+          <t>Hacha</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3192,52 +3182,52 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>bloqueo +2</t>
+          <t>Rompe armadura.</t>
         </is>
       </c>
       <c r="I21" t="n">
         <v>6</v>
       </c>
       <c r="J21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="n">
-        <v>10</v>
-      </c>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
-        <v>1</v>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>new-martillo-de-guerra-runico</t>
+          <t>new-horquilla</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Martillo de guerra rúnico</t>
+          <t>Horquilla</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3246,32 +3236,30 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>170</v>
+        <v>50</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>25% de chances de dejar en pajaritos</t>
+          <t>rango +1</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="n">
-        <v>1</v>
-      </c>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
@@ -3279,17 +3267,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>new-espada-bastarda</t>
+          <t>new-lanza-corta</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Espada bastarda</t>
+          <t>Lanza corta</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3304,15 +3292,15 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>parry+1, bloqueo+1</t>
+          <t>rango +1</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -3329,17 +3317,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>new-estoque-de-duelista</t>
+          <t>cat-machete</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Estoque de duelista</t>
+          <t>Machete</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3354,44 +3342,46 @@
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>165</v>
+        <v>55</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Ingora 2 de resistencia al crítico</t>
+          <t>+10% de daño crítico</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
-      <c r="M24" t="n">
-        <v>1</v>
-      </c>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cat-hacha-de-mano</t>
+          <t>cat-maza</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Hacha de doble filo</t>
+          <t>Maza</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3400,24 +3390,24 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>120</v>
+        <v>66</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Rompe armadura. Ignora 1 resistencia al crítico</t>
+          <t>Bloqueo +1</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -3435,17 +3425,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cat-mangual</t>
+          <t>new-maza-de-guardia</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mangual</t>
+          <t>Maza de guardia</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3454,24 +3444,24 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Alcance +1.</t>
+          <t>Bloqueo +1</t>
         </is>
       </c>
       <c r="I26" t="n">
         <v>8</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
@@ -3480,26 +3470,22 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>new-punal-aserrado</t>
+          <t>new-pica-hielos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Puñal aserrado</t>
+          <t>Pica Hielos</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3511,16 +3497,12 @@
         <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Rompe armadura.</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
         <v>2</v>
       </c>
@@ -3536,8 +3518,624 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>new-colmillo-dientes-de-sable</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Colmillo dientes de sable</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>150</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Deja sangrando x2hp</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>new-espadon</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Espadón</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>140</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>bloqueo +2</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>6</v>
+      </c>
+      <c r="J29" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>10</v>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="n">
+        <v>1</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>new-martillo-de-guerra-runico</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Martillo de guerra rúnico</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>170</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>25% de chances de dejar en pajaritos</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>8</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="n">
+        <v>1</v>
+      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>new-punal-de-dorne</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Puñal de Dorne</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>150</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Veneno stock 4</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>new-aguijon-de-manticora</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Aguijón de mantícora</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>500</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>critico +2, dza +2, 50% de chance de stunear</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>new-aguijon-de-esgrima</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Aguijón de esgrima</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>110</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>parry +2, pdg +1</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>2</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>new-espada-bastarda</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Espada bastarda</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>120</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>parry+1, bloqueo+1</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>4</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>new-estoque-de-duelista</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Estoque de duelista</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>80</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Ingora 2 de resistencia al crítico</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>2</v>
+      </c>
+      <c r="J35" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>1</v>
+      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>cat-hacha-de-mano</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Hacha de doble filo</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="n">
+        <v>120</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Rompe armadura. Ignora 1 resistencia al crítico</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>6</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>new-lanza-militar</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Lanza militar</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>80</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Daño amplificado.</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>2</v>
+      </c>
+      <c r="J37" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>cat-mangual</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Mangual</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>120</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Alcance +1.</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>8</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>new-punal-aserrado</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Puñal aserrado</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>100</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Rompe armadura.</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>2</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R27"/>
+  <autoFilter ref="A1:R39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3548,7 +4146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3666,12 +4264,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>new-escudo-de-acero-laminado</t>
+          <t>new-broquel-de-hierro</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Escudo de acero laminado</t>
+          <t>Broquel de hierro</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3685,39 +4283,45 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>87</v>
-      </c>
-      <c r="H2" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>parry +2, resistencia a críticos tipo 4</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
-        <v>1</v>
-      </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="n">
+        <v>2</v>
+      </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cat-escudo-grande</t>
+          <t>new-escudo-de-acero-laminado</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Escudo grande</t>
+          <t>Escudo de acero laminado</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3731,47 +4335,39 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>82</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>+2 al bloqueo</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>6</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
         <v>7</v>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cat-escudo-pav-s</t>
+          <t>new-escudo-de-escamas</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Escudo pavés</t>
+          <t>Escudo de escamas</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3785,22 +4381,20 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>116</v>
+        <v>90</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>+1 a estabilidad, +1 al bloqueo</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>6</v>
-      </c>
+          <t>Resistencia a críticos tipo 6 y 8</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
         <v>6</v>
       </c>
@@ -3811,21 +4405,17 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cat-escudo-romano</t>
+          <t>cat-escudo-grande</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Escudo romano</t>
+          <t>Escudo grande</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3835,28 +4425,26 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>escudo_2m</t>
+          <t>escudo_1m</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>131</v>
+        <v>90</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>+4 al bloqueo. Movimiento y ataque lento</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>6</v>
-      </c>
+          <t>bloqueo +2</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
@@ -3864,7 +4452,11 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>bloqueo:2</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>sí</t>
@@ -3874,12 +4466,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cat-escudo-triangular</t>
+          <t>cat-escudo-romano</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Escudo triangular</t>
+          <t>Escudo romano</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3893,24 +4485,22 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>+2 al bloqueo</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>6</v>
-      </c>
+          <t>bloqueo +3</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
@@ -3918,7 +4508,11 @@
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>bloqueo:3</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>sí</t>
@@ -3928,17 +4522,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cat-broquel</t>
+          <t>cat-escudo-triangular</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Broquel</t>
+          <t>Escudo triangular</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3947,24 +4541,22 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>42</v>
+        <v>110</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>+2 a estabilidad</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
+          <t>bloqueo +2</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="n">
         <v>6</v>
-      </c>
-      <c r="J7" t="n">
-        <v>3</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
@@ -3982,12 +4574,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cat-escudo-peque-o</t>
+          <t>cat-broquel</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Escudo pequeño</t>
+          <t>Broquel de bronce</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4001,31 +4593,31 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>+1 al bloqueo, +1 a la estabilidad</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>6</v>
-      </c>
+          <t>parry +1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="P8" t="n">
+        <v>1</v>
+      </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
@@ -4036,12 +4628,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>new-rodela-de-cuero</t>
+          <t>new-escudo-de-asalto</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rodela de cuero</t>
+          <t>Escudo de asalto</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4055,22 +4647,24 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>42</v>
-      </c>
-      <c r="H9" t="inlineStr"/>
+        <v>70</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>bloqueo +2</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" t="n">
-        <v>1</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -4082,12 +4676,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>new-tapa-de-tacho-de-basura-reforzada</t>
+          <t>new-escudo-de-cuero-endurecido</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tapa de tacho de basura reforzada</t>
+          <t>Escudo de cuero endurecido</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4101,15 +4695,19 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>46</v>
-      </c>
-      <c r="H10" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Resistencia a críticos tipo 2 y 4</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
         <v>4</v>
@@ -4117,9 +4715,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
-        <v>1</v>
-      </c>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
@@ -4128,17 +4724,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>new-egida-menor</t>
+          <t>new-escudo-de-madera</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Égida menor</t>
+          <t>Escudo de madera</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4147,38 +4743,728 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>326</v>
+        <v>70</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Al bloquear un golpe crítico, cura 10 HP instantáneos al portador.</t>
+          <t>Resistencia a críticos tipo 4 y 6</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>1</v>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="n">
-        <v>1</v>
-      </c>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>cat-escudo-peque-o</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Escudo pequeño</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>46</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Resistencia +1 a tipos 4, 6 y 8</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>new-rodela-de-cuero</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rodela de cuero</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>40</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Resistencia a críticos tipo 2</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>new-tapa-de-tacho-de-basura-reforzada</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Rodela de madera</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>60</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Resistencia a críticos tipo 4 y 6</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>new-tapa-de-tacho-de-basura</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tapa de tacho de basura</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>60</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Resistencia a críticos tipo 8</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>new-broquel-de-titanio</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Broquel de titanio</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>190</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Parry +3, bloqueo +1, resistencia a críticos tipo 2 y 4</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="n">
+        <v>7</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>new-rodela-de-cobra</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Rodela de cobra</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>220</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>parry +2, bloqueo +1. Si bloquea con exito, +2 a pg en próximo ataque</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>new-egida-de-gladiador</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Égida de Gladiador</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>250</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>bloqueo +4, +1 a resistencia de todo crítico</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>8</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>bloqueo:4</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>new-escudo-de-shiryu</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Escudo de ShiRyu</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>600</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>parry  +4, bloqueo +4, inmuniza ruptura de armadura</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>10</v>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>new-broquel-de-acero</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Broquel de acero</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>120</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Parry +3, resistencia a críticos tipo 2 y 4</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>new-escudo-de-torre</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Escudo de torre</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>140</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>parry +1, bloqueo +3</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
+        <v>9</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>bloqueo:3</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cat-escudo-pav-s</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Escudo pavés</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>90</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Bloqueo +1, Resistencia crit tipo 8 y 10</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>7</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>bloqueo:1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>new-escudo-triangular</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Escudo triangular</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>160</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>bloqueo +2, Resistencia a críticos 4, 6 y 8</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>8</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>new-egida-menor</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Égida menor</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>escudo_1m</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>130</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Resistencia a todos los críticos +1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="n">
+        <v>6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
+      <c r="O24" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R11"/>
+  <autoFilter ref="A1:R24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9324,7 +10610,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>26 ítems</t>
+          <t>38 ítems</t>
         </is>
       </c>
     </row>
@@ -9336,7 +10622,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>10 ítems</t>
+          <t>23 ítems</t>
         </is>
       </c>
     </row>
@@ -9372,7 +10658,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>134 ítems</t>
+          <t>159 ítems</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catálogo: 162 ítems (4 armas nuevas del Excel)
Entran Cimitarra, Hoz, Machete y Sable; el Machete viejo sale, reemplazado
por el nuevo. Se ajustan Espada ancha y Espada corta de instrucción.

El Excel queda regenerado con los IDs ya puestos, para que la próxima
edición no los duplique.
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Consumibles'!$A$1:$S$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$R$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$R$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Escudos'!$A$1:$R$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defensivos'!$A$1:$AE$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Otros'!$A$1:$Q$2</definedName>
@@ -2069,7 +2069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R39"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2308,7 +2308,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -2923,12 +2923,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>new-cuchillo-de-cazador</t>
+          <t>new-cimitarra</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cuchillo de cazador</t>
+          <t>Cimitarra</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2945,14 +2945,18 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>30</v>
-      </c>
-      <c r="H16" t="inlineStr"/>
+        <v>55</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>parry +1</t>
+        </is>
+      </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -2960,7 +2964,9 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
@@ -2969,12 +2975,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>new-daga</t>
+          <t>new-cuchillo-de-cazador</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Daga</t>
+          <t>Cuchillo de cazador</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2991,17 +2997,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
         <v>2</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -3015,12 +3021,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cat-espada-corta</t>
+          <t>new-daga</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Espada corta</t>
+          <t>Daga</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3037,17 +3043,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -3056,21 +3062,17 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>new-espada-corta-de-instruccion</t>
+          <t>cat-espada-corta</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Espada corta de instrucción</t>
+          <t>Espada corta</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3084,13 +3086,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
@@ -3100,25 +3102,27 @@
         <v>0</v>
       </c>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="n">
-        <v>10</v>
-      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>new-estileto-comun</t>
+          <t>new-espada-corta-de-instruccion</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Estileto común</t>
+          <t>Espada corta de instrucción</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3132,21 +3136,17 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
         <v>50</v>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>crítico +1</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -3163,12 +3163,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cat-hacha</t>
+          <t>new-estileto-comun</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hacha</t>
+          <t>Estileto común</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3185,18 +3185,18 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Rompe armadura.</t>
+          <t>crítico +1</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -3208,21 +3208,17 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>new-horquilla</t>
+          <t>cat-hacha</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Horquilla</t>
+          <t>Hacha</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3239,18 +3235,18 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>rango +1</t>
+          <t>Rompe armadura.</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -3262,17 +3258,21 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>new-lanza-corta</t>
+          <t>new-horquilla</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Lanza corta</t>
+          <t>Horquilla</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3286,13 +3286,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -3317,12 +3317,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cat-machete</t>
+          <t>new-hoz</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Machete</t>
+          <t>Hoz</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3339,16 +3339,12 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>55</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>+10% de daño crítico</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
         <v>4</v>
       </c>
@@ -3362,21 +3358,17 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cat-maza</t>
+          <t>new-lanza-corta</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Maza</t>
+          <t>Lanza corta</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3393,21 +3385,21 @@
         <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Bloqueo +1</t>
+          <t>rango +1</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -3416,21 +3408,17 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>new-maza-de-guardia</t>
+          <t>new-machete</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Maza de guardia</t>
+          <t>Machete</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3444,21 +3432,21 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Bloqueo +1</t>
+          <t>romper armadura 50%</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -3475,12 +3463,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>new-pica-hielos</t>
+          <t>cat-maza</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Pica Hielos</t>
+          <t>Maza</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3500,14 +3488,18 @@
         <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>40</v>
-      </c>
-      <c r="H27" t="inlineStr"/>
+        <v>66</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Bloqueo +1</t>
+        </is>
+      </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
@@ -3516,22 +3508,26 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>new-colmillo-dientes-de-sable</t>
+          <t>new-maza-de-guardia</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Colmillo dientes de sable</t>
+          <t>Maza de guardia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3540,24 +3536,24 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>150</v>
+        <v>55</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Deja sangrando x2hp</t>
+          <t>Bloqueo +1</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -3571,17 +3567,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>new-espadon</t>
+          <t>new-pica-hielos</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Espadón</t>
+          <t>Pica Hielos</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3590,33 +3586,25 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>140</v>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>bloqueo +2</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="n">
-        <v>10</v>
-      </c>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="n">
-        <v>1</v>
-      </c>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
@@ -3625,17 +3613,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>new-martillo-de-guerra-runico</t>
+          <t>new-sable</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Martillo de guerra rúnico</t>
+          <t>Sable</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3644,32 +3632,30 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>170</v>
+        <v>40</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>25% de chances de dejar en pajaritos</t>
+          <t>iniciativa +1</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J30" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
-      <c r="O30" t="n">
-        <v>1</v>
-      </c>
+      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
@@ -3677,12 +3663,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>new-punal-de-dorne</t>
+          <t>new-colmillo-dientes-de-sable</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Puñal de Dorne</t>
+          <t>Colmillo dientes de sable</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3706,14 +3692,14 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Veneno stock 4</t>
+          <t>Deja sangrando x2hp</t>
         </is>
       </c>
       <c r="I31" t="n">
         <v>2</v>
       </c>
       <c r="J31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -3727,17 +3713,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>new-aguijon-de-manticora</t>
+          <t>new-espadon</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Aguijón de mantícora</t>
+          <t>Espadón</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Legendario</t>
+          <t>Excepcional</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3746,29 +3732,33 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>500</v>
+        <v>140</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>critico +2, dza +2, 50% de chance de stunear</t>
+          <t>bloqueo +2</t>
         </is>
       </c>
       <c r="I32" t="n">
+        <v>6</v>
+      </c>
+      <c r="J32" t="n">
         <v>2</v>
       </c>
-      <c r="J32" t="n">
-        <v>0</v>
-      </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>10</v>
+      </c>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" t="n">
+        <v>1</v>
+      </c>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
@@ -3777,17 +3767,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>new-aguijon-de-esgrima</t>
+          <t>new-martillo-de-guerra-runico</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Aguijón de esgrima</t>
+          <t>Martillo de guerra rúnico</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Excepcional</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3796,30 +3786,32 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>110</v>
+        <v>170</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>parry +2, pdg +1</t>
+          <t>25% de chances de dejar en pajaritos</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="n">
+        <v>1</v>
+      </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
@@ -3827,17 +3819,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>new-espada-bastarda</t>
+          <t>new-punal-de-dorne</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Espada bastarda</t>
+          <t>Puñal de Dorne</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Excepcional</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3852,18 +3844,18 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>parry+1, bloqueo+1</t>
+          <t>Veneno stock 4</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -3877,17 +3869,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>new-estoque-de-duelista</t>
+          <t>new-aguijon-de-manticora</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Estoque de duelista</t>
+          <t>Aguijón de mantícora</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Legendario</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3896,30 +3888,28 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>80</v>
+        <v>500</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Ingora 2 de resistencia al crítico</t>
+          <t>critico +2, dza +2, 50% de chance de stunear</t>
         </is>
       </c>
       <c r="I35" t="n">
         <v>2</v>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
-      <c r="M35" t="n">
-        <v>1</v>
-      </c>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
@@ -3929,12 +3919,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cat-hacha-de-mano</t>
+          <t>new-aguijon-de-esgrima</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hacha de doble filo</t>
+          <t>Aguijón de esgrima</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3948,21 +3938,21 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Rompe armadura. Ignora 1 resistencia al crítico</t>
+          <t>parry +2, pdg +1</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -3974,21 +3964,17 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>new-lanza-militar</t>
+          <t>new-espada-bastarda</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Lanza militar</t>
+          <t>Espada bastarda</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4008,18 +3994,18 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Daño amplificado.</t>
+          <t>parry+1, bloqueo+1</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -4033,12 +4019,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>cat-mangual</t>
+          <t>new-estoque-de-duelista</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mangual</t>
+          <t>Estoque de duelista</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4052,47 +4038,45 @@
         </is>
       </c>
       <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>80</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Ingora 2 de resistencia al crítico</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
         <v>2</v>
       </c>
-      <c r="F38" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" t="n">
-        <v>120</v>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Alcance +1.</t>
-        </is>
-      </c>
-      <c r="I38" t="n">
-        <v>8</v>
-      </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>1</v>
+      </c>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>new-punal-aserrado</t>
+          <t>cat-hacha-de-mano</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Puñal aserrado</t>
+          <t>Hacha de doble filo</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4106,21 +4090,21 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Rompe armadura.</t>
+          <t>Rompe armadura. Ignora 1 resistencia al crítico</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -4132,10 +4116,168 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>new-lanza-militar</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Lanza militar</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>80</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Daño amplificado.</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" t="n">
+        <v>2</v>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>cat-mangual</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Mangual</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>120</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Alcance +1.</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>8</v>
+      </c>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>new-punal-aserrado</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Puñal aserrado</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>100</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Rompe armadura.</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>2</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R39"/>
+  <autoFilter ref="A1:R42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10610,7 +10752,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>38 ítems</t>
+          <t>41 ítems</t>
         </is>
       </c>
     </row>
@@ -10658,7 +10800,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>159 ítems</t>
+          <t>162 ítems</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ficha: un ítem puede aplicar un estado mientras está equipado
Los Guantes de piel de troll prometían regeneración "a aplicar a mano".
Ahora, al ponérselos, aparece solo el estado que la otorga, y al sacárselos
se va con ellos.

Está hecho general, no para ese ítem: cualquiera puede declarar un estado
al equipar desde el Excel, con sus columnas Estado al equipar, HP por turno
equipado y Detalle del estado equipado.

El estado se distingue de los que carga el jugador —lleva el engranaje y el
borde verde— y no se puede duplicar. Si lo pausa, se respeta: no se
reactiva solo. Si lo borra teniendo el ítem puesto, vuelve, porque lo
genera el ítem y no él.
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -16,9 +16,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Consumibles'!$A$1:$S$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$R$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Escudos'!$A$1:$R$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defensivos'!$A$1:$AE$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$U$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Escudos'!$A$1:$U$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defensivos'!$A$1:$AH$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Otros'!$A$1:$Q$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -621,17 +621,9 @@
       <c r="I2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -676,18 +668,9 @@
       <c r="I3" t="n">
         <v>1</v>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -727,17 +710,9 @@
       <c r="I4" t="n">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
           <t>sí</t>
@@ -782,17 +757,9 @@
       <c r="I5" t="n">
         <v>1</v>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
           <t>sí</t>
@@ -837,17 +804,9 @@
       <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
         <v>0</v>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
           <t>sí</t>
@@ -892,17 +851,9 @@
       <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
           <t>sí</t>
@@ -947,17 +898,9 @@
       <c r="I8" t="n">
         <v>1</v>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1002,17 +945,9 @@
       <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1057,19 +992,12 @@
       <c r="I10" t="n">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>50</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1114,19 +1042,12 @@
       <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>100</v>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1171,11 +1092,9 @@
       <c r="I12" t="n">
         <v>1</v>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>Regeneración (poción)</t>
@@ -1187,9 +1106,6 @@
       <c r="O12" t="n">
         <v>20</v>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1234,17 +1150,9 @@
       <c r="I13" t="n">
         <v>5</v>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1289,17 +1197,9 @@
       <c r="I14" t="n">
         <v>1</v>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="n">
         <v>0</v>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1344,17 +1244,9 @@
       <c r="I15" t="n">
         <v>1</v>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1399,17 +1291,9 @@
       <c r="I16" t="n">
         <v>1</v>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
         <v>0</v>
       </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1454,17 +1338,9 @@
       <c r="I17" t="n">
         <v>1</v>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
         <v>25</v>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1509,11 +1385,9 @@
       <c r="I18" t="n">
         <v>1</v>
       </c>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
         <v>0</v>
       </c>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>Regeneración (poción)</t>
@@ -1525,9 +1399,6 @@
       <c r="O18" t="n">
         <v>10</v>
       </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1572,17 +1443,9 @@
       <c r="I19" t="n">
         <v>2</v>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
         <v>0</v>
       </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1619,22 +1482,12 @@
       <c r="G20" t="n">
         <v>10</v>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
         <v>1</v>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
         <v>10</v>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1680,13 +1533,6 @@
       <c r="K21" t="n">
         <v>100</v>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1737,7 +1583,6 @@
       <c r="K22" t="n">
         <v>0</v>
       </c>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>Regeneración (poción)</t>
@@ -1749,9 +1594,6 @@
       <c r="O22" t="n">
         <v>20</v>
       </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1796,17 +1638,9 @@
       <c r="I23" t="n">
         <v>1</v>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="n">
         <v>0</v>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1857,13 +1691,6 @@
       <c r="K24" t="n">
         <v>25</v>
       </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1908,17 +1735,9 @@
       <c r="I25" t="n">
         <v>1</v>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
         <v>100</v>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
           <t>sí</t>
@@ -1969,7 +1788,6 @@
       <c r="K26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>Regeneración (poción)</t>
@@ -1981,9 +1799,6 @@
       <c r="O26" t="n">
         <v>10</v>
       </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
           <t>sí</t>
@@ -2028,18 +1843,14 @@
       <c r="I27" t="n">
         <v>1</v>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>Polilla revoloteando</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>sí</t>
@@ -2050,7 +1861,6 @@
           <t>La polilla revolotea a tu alrededor. Cuando quieras, gastala para sumar +2 a una tirada de dado: borrá este estado en ese momento para marcar que ya la usaste. Hasta entonces queda acá, sin vencerse.</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
           <t>sí</t>
@@ -2069,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:U42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2088,8 +1898,11 @@
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2175,10 +1988,25 @@
       </c>
       <c r="Q1" s="2" t="inlineStr">
         <is>
+          <t>Estado al equipar</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>HP por turno equipado</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Detalle del estado equipado</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
           <t>Otros modificadores</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Tiene imagen</t>
         </is>
@@ -2228,13 +2056,6 @@
       <c r="K2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2277,14 +2098,6 @@
       <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2327,14 +2140,7 @@
       <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -2384,13 +2190,7 @@
       <c r="K5" t="n">
         <v>1</v>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -2437,14 +2237,6 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2487,16 +2279,10 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
         <v>1</v>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -2543,16 +2329,10 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -2599,14 +2379,6 @@
       <c r="J9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2649,14 +2421,7 @@
       <c r="J10" t="n">
         <v>3</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -2703,18 +2468,12 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>10</v>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
         <v>1</v>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2757,14 +2516,6 @@
       <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2807,14 +2558,7 @@
       <c r="J13" t="n">
         <v>0</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -2850,7 +2594,6 @@
       <c r="G14" t="n">
         <v>87</v>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
         <v>6</v>
       </c>
@@ -2860,13 +2603,6 @@
       <c r="K14" t="n">
         <v>1</v>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2909,16 +2645,9 @@
       <c r="J15" t="n">
         <v>0</v>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>10</v>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2961,16 +2690,9 @@
       <c r="J16" t="n">
         <v>0</v>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
         <v>1</v>
       </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3002,21 +2724,12 @@
       <c r="G17" t="n">
         <v>30</v>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
         <v>2</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3048,21 +2761,12 @@
       <c r="G18" t="n">
         <v>40</v>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
         <v>2</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3094,21 +2798,13 @@
       <c r="G19" t="n">
         <v>30</v>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
         <v>4</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -3144,21 +2840,12 @@
       <c r="G20" t="n">
         <v>50</v>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
         <v>4</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3201,14 +2888,6 @@
       <c r="J21" t="n">
         <v>0</v>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3251,14 +2930,7 @@
       <c r="J22" t="n">
         <v>0</v>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -3305,14 +2977,6 @@
       <c r="J23" t="n">
         <v>0</v>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3344,21 +3008,12 @@
       <c r="G24" t="n">
         <v>0</v>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
         <v>4</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3401,14 +3056,6 @@
       <c r="J25" t="n">
         <v>0</v>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3451,14 +3098,6 @@
       <c r="J26" t="n">
         <v>0</v>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3501,14 +3140,7 @@
       <c r="J27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -3555,14 +3187,6 @@
       <c r="J28" t="n">
         <v>0</v>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3594,21 +3218,12 @@
       <c r="G29" t="n">
         <v>40</v>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
         <v>2</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3651,14 +3266,6 @@
       <c r="J30" t="n">
         <v>0</v>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3701,14 +3308,6 @@
       <c r="J31" t="n">
         <v>1</v>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3751,18 +3350,12 @@
       <c r="J32" t="n">
         <v>2</v>
       </c>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
         <v>10</v>
       </c>
-      <c r="M32" t="inlineStr"/>
       <c r="N32" t="n">
         <v>1</v>
       </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3805,16 +3398,9 @@
       <c r="J33" t="n">
         <v>3</v>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
       <c r="O33" t="n">
         <v>1</v>
       </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3857,14 +3443,6 @@
       <c r="J34" t="n">
         <v>2</v>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3907,14 +3485,6 @@
       <c r="J35" t="n">
         <v>0</v>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3957,14 +3527,6 @@
       <c r="J36" t="n">
         <v>0</v>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4007,14 +3569,6 @@
       <c r="J37" t="n">
         <v>0</v>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4057,16 +3611,9 @@
       <c r="J38" t="n">
         <v>2</v>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="n">
         <v>1</v>
       </c>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4109,14 +3656,7 @@
       <c r="J39" t="n">
         <v>0</v>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -4163,14 +3703,6 @@
       <c r="J40" t="n">
         <v>2</v>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4213,14 +3745,7 @@
       <c r="J41" t="n">
         <v>1</v>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -4267,17 +3792,9 @@
       <c r="J42" t="n">
         <v>0</v>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R42"/>
+  <autoFilter ref="A1:U42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4288,7 +3805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4307,8 +3824,11 @@
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4394,10 +3914,25 @@
       </c>
       <c r="Q1" s="2" t="inlineStr">
         <is>
+          <t>Estado al equipar</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>HP por turno equipado</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Detalle del estado equipado</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
           <t>Otros modificadores</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Tiene imagen</t>
         </is>
@@ -4438,22 +3973,15 @@
           <t>parry +2, resistencia a críticos tipo 4</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
         <v>4</v>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>1</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>2</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4485,21 +4013,12 @@
       <c r="G3" t="n">
         <v>90</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
         <v>7</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4536,18 +4055,9 @@
           <t>Resistencia a críticos tipo 6 y 8</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
         <v>6</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4584,22 +4094,15 @@
           <t>bloqueo +2</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
         <v>7</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>bloqueo:2</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -4640,22 +4143,15 @@
           <t>bloqueo +3</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
         <v>10</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>bloqueo:3</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -4696,18 +4192,10 @@
           <t>bloqueo +2</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
         <v>6</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -4748,20 +4236,13 @@
           <t>parry +1</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
         <v>3</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -4802,18 +4283,9 @@
           <t>bloqueo +2</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
         <v>4</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4850,18 +4322,9 @@
           <t>Resistencia a críticos tipo 2 y 4</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
         <v>4</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4898,22 +4361,15 @@
           <t>Resistencia a críticos tipo 4 y 6</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
         <v>5</v>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>1</v>
       </c>
       <c r="M11" t="n">
         <v>1</v>
       </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4950,11 +4406,9 @@
           <t>Resistencia +1 a tipos 4, 6 y 8</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
         <v>4</v>
       </c>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>1</v>
       </c>
@@ -4964,10 +4418,7 @@
       <c r="N12" t="n">
         <v>1</v>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -5008,20 +4459,12 @@
           <t>Resistencia a críticos tipo 2</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
         <v>3</v>
       </c>
       <c r="K13" t="n">
         <v>1</v>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5058,11 +4501,9 @@
           <t>Resistencia a críticos tipo 4 y 6</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="n">
         <v>4</v>
       </c>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>1</v>
       </c>
@@ -5072,10 +4513,6 @@
       <c r="N14" t="n">
         <v>1</v>
       </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5112,18 +4549,9 @@
           <t>Resistencia a críticos tipo 8</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
         <v>3</v>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5160,18 +4588,9 @@
           <t>Parry +3, bloqueo +1, resistencia a críticos tipo 2 y 4</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
         <v>7</v>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5208,18 +4627,9 @@
           <t>parry +2, bloqueo +1. Si bloquea con exito, +2 a pg en próximo ataque</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
         <v>4</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5256,7 +4666,6 @@
           <t>bloqueo +4, +1 a resistencia de todo crítico</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="n">
         <v>8</v>
       </c>
@@ -5278,12 +4687,11 @@
       <c r="P18" t="n">
         <v>2</v>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>bloqueo:4</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5320,18 +4728,9 @@
           <t>parry  +4, bloqueo +4, inmuniza ruptura de armadura</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="n">
         <v>10</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5368,7 +4767,6 @@
           <t>Parry +3, resistencia a críticos tipo 2 y 4</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
         <v>5</v>
       </c>
@@ -5378,12 +4776,6 @@
       <c r="L20" t="n">
         <v>1</v>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5420,24 +4812,17 @@
           <t>parry +1, bloqueo +3</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="n">
         <v>9</v>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>1</v>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>bloqueo:3</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5474,26 +4859,21 @@
           <t>Bloqueo +1, Resistencia crit tipo 8 y 10</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="n">
         <v>7</v>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
         <v>1</v>
       </c>
       <c r="O22" t="n">
         <v>1</v>
       </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>bloqueo:1</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -5534,18 +4914,9 @@
           <t>bloqueo +2, Resistencia a críticos 4, 6 y 8</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
         <v>8</v>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5582,7 +4953,6 @@
           <t>Resistencia a todos los críticos +1</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
         <v>6</v>
       </c>
@@ -5601,12 +4971,9 @@
       <c r="O24" t="n">
         <v>1</v>
       </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R24"/>
+  <autoFilter ref="A1:U24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5617,7 +4984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE73"/>
+  <dimension ref="A1:AH73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5649,8 +5016,11 @@
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="13" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
-    <col width="30" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="30" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5801,10 +5171,25 @@
       </c>
       <c r="AD1" s="2" t="inlineStr">
         <is>
+          <t>Estado al equipar</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>HP por turno equipado</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>Detalle del estado equipado</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
           <t>Otros modificadores</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Tiene imagen</t>
         </is>
@@ -5854,26 +5239,6 @@
       <c r="K2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5919,28 +5284,9 @@
       <c r="K3" t="n">
         <v>1</v>
       </c>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>1</v>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5972,36 +5318,15 @@
       <c r="G4" t="n">
         <v>92</v>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
         <v>4</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>1</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
         <v>1</v>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6033,36 +5358,15 @@
       <c r="G5" t="n">
         <v>93</v>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
         <v>6</v>
       </c>
       <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>1</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6094,36 +5398,15 @@
       <c r="G6" t="n">
         <v>106</v>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>7</v>
       </c>
       <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
         <v>1</v>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6172,25 +5455,6 @@
       <c r="L7" t="n">
         <v>1</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6222,36 +5486,15 @@
       <c r="G8" t="n">
         <v>98</v>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
         <v>6</v>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
         <v>1</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6291,32 +5534,12 @@
       <c r="I9" t="n">
         <v>6</v>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>1</v>
       </c>
       <c r="M9" t="n">
         <v>1</v>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6365,25 +5588,6 @@
       <c r="L10" t="n">
         <v>1</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6423,32 +5627,12 @@
       <c r="I11" t="n">
         <v>4</v>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6494,26 +5678,6 @@
       <c r="K12" t="n">
         <v>1</v>
       </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6556,29 +5720,9 @@
       <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
       <c r="S13" t="n">
         <v>1</v>
       </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6618,32 +5762,12 @@
       <c r="I14" t="n">
         <v>5</v>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="n">
         <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr"/>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6683,34 +5807,15 @@
       <c r="I15" t="n">
         <v>2</v>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>1</v>
       </c>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="n">
         <v>1</v>
       </c>
       <c r="AA15" t="n">
         <v>1</v>
       </c>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6756,26 +5861,6 @@
       <c r="K16" t="n">
         <v>1</v>
       </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6815,32 +5900,12 @@
       <c r="I17" t="n">
         <v>4</v>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>1</v>
       </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
         <v>1</v>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
-      <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6872,36 +5937,15 @@
       <c r="G18" t="n">
         <v>111</v>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
         <v>7</v>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6941,7 +5985,6 @@
       <c r="I19" t="n">
         <v>6</v>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
         <v>1</v>
       </c>
@@ -6951,26 +5994,9 @@
       <c r="M19" t="n">
         <v>1</v>
       </c>
-      <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
         <v>-1</v>
       </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7002,36 +6028,15 @@
       <c r="G20" t="n">
         <v>92</v>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
         <v>4</v>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
         <v>1</v>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="n">
         <v>1</v>
       </c>
-      <c r="AC20" t="inlineStr"/>
-      <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7074,31 +6079,12 @@
       <c r="J21" t="n">
         <v>1</v>
       </c>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
-      <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr"/>
-      <c r="AC21" t="inlineStr"/>
-      <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7130,36 +6116,15 @@
       <c r="G22" t="n">
         <v>98</v>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
         <v>6</v>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
         <v>1</v>
       </c>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
         <v>1</v>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7199,32 +6164,12 @@
       <c r="I23" t="n">
         <v>5</v>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
       </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
-      <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7267,27 +6212,6 @@
       <c r="J24" t="n">
         <v>1</v>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
-      <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7319,34 +6243,12 @@
       <c r="G25" t="n">
         <v>37</v>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
         <v>3</v>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
         <v>1</v>
       </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
-      <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7378,34 +6280,12 @@
       <c r="G26" t="n">
         <v>41</v>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
         <v>4</v>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
         <v>1</v>
       </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="inlineStr"/>
-      <c r="AA26" t="inlineStr"/>
-      <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="inlineStr"/>
-      <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7437,34 +6317,12 @@
       <c r="G27" t="n">
         <v>38</v>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
         <v>2</v>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
       <c r="O27" t="n">
         <v>1</v>
       </c>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
-      <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="inlineStr"/>
-      <c r="AD27" t="inlineStr"/>
-      <c r="AE27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7504,30 +6362,9 @@
       <c r="I28" t="n">
         <v>3</v>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
         <v>1</v>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr"/>
-      <c r="AB28" t="inlineStr"/>
-      <c r="AC28" t="inlineStr"/>
-      <c r="AD28" t="inlineStr"/>
-      <c r="AE28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7559,34 +6396,12 @@
       <c r="G29" t="n">
         <v>32</v>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
         <v>2</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr"/>
-      <c r="AB29" t="inlineStr"/>
-      <c r="AC29" t="inlineStr"/>
-      <c r="AD29" t="inlineStr"/>
-      <c r="AE29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7618,34 +6433,12 @@
       <c r="G30" t="n">
         <v>42</v>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="n">
         <v>3</v>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
         <v>1</v>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
-      <c r="AA30" t="inlineStr"/>
-      <c r="AB30" t="inlineStr"/>
-      <c r="AC30" t="inlineStr"/>
-      <c r="AD30" t="inlineStr"/>
-      <c r="AE30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7677,34 +6470,12 @@
       <c r="G31" t="n">
         <v>42</v>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
         <v>3</v>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
         <v>1</v>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="inlineStr"/>
-      <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="inlineStr"/>
-      <c r="AD31" t="inlineStr"/>
-      <c r="AE31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7736,34 +6507,12 @@
       <c r="G32" t="n">
         <v>37</v>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="n">
         <v>3</v>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
         <v>1</v>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="inlineStr"/>
-      <c r="AB32" t="inlineStr"/>
-      <c r="AC32" t="inlineStr"/>
-      <c r="AD32" t="inlineStr"/>
-      <c r="AE32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7795,34 +6544,12 @@
       <c r="G33" t="n">
         <v>37</v>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
         <v>2</v>
       </c>
       <c r="J33" t="n">
         <v>1</v>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="inlineStr"/>
-      <c r="AB33" t="inlineStr"/>
-      <c r="AC33" t="inlineStr"/>
-      <c r="AD33" t="inlineStr"/>
-      <c r="AE33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7862,30 +6589,9 @@
       <c r="I34" t="n">
         <v>3</v>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="n">
         <v>1</v>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr"/>
-      <c r="Y34" t="inlineStr"/>
-      <c r="Z34" t="inlineStr"/>
-      <c r="AA34" t="inlineStr"/>
-      <c r="AB34" t="inlineStr"/>
-      <c r="AC34" t="inlineStr"/>
-      <c r="AD34" t="inlineStr"/>
-      <c r="AE34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7917,34 +6623,12 @@
       <c r="G35" t="n">
         <v>56</v>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="n">
         <v>5</v>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="n">
         <v>1</v>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
-      <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
-      <c r="X35" t="inlineStr"/>
-      <c r="Y35" t="inlineStr"/>
-      <c r="Z35" t="inlineStr"/>
-      <c r="AA35" t="inlineStr"/>
-      <c r="AB35" t="inlineStr"/>
-      <c r="AC35" t="inlineStr"/>
-      <c r="AD35" t="inlineStr"/>
-      <c r="AE35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7976,34 +6660,12 @@
       <c r="G36" t="n">
         <v>59</v>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="n">
         <v>6</v>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
       <c r="M36" t="n">
         <v>1</v>
       </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr"/>
-      <c r="X36" t="inlineStr"/>
-      <c r="Y36" t="inlineStr"/>
-      <c r="Z36" t="inlineStr"/>
-      <c r="AA36" t="inlineStr"/>
-      <c r="AB36" t="inlineStr"/>
-      <c r="AC36" t="inlineStr"/>
-      <c r="AD36" t="inlineStr"/>
-      <c r="AE36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8035,34 +6697,12 @@
       <c r="G37" t="n">
         <v>42</v>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="n">
         <v>3</v>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
       <c r="M37" t="n">
         <v>1</v>
       </c>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
-      <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr"/>
-      <c r="Z37" t="inlineStr"/>
-      <c r="AA37" t="inlineStr"/>
-      <c r="AB37" t="inlineStr"/>
-      <c r="AC37" t="inlineStr"/>
-      <c r="AD37" t="inlineStr"/>
-      <c r="AE37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8094,34 +6734,12 @@
       <c r="G38" t="n">
         <v>46</v>
       </c>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="n">
         <v>4</v>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="n">
         <v>1</v>
       </c>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="inlineStr"/>
-      <c r="Z38" t="inlineStr"/>
-      <c r="AA38" t="inlineStr"/>
-      <c r="AB38" t="inlineStr"/>
-      <c r="AC38" t="inlineStr"/>
-      <c r="AD38" t="inlineStr"/>
-      <c r="AE38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8161,32 +6779,12 @@
       <c r="I39" t="n">
         <v>3</v>
       </c>
-      <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
         <v>1</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr"/>
-      <c r="Z39" t="inlineStr"/>
-      <c r="AA39" t="inlineStr"/>
-      <c r="AB39" t="inlineStr"/>
-      <c r="AC39" t="inlineStr"/>
-      <c r="AD39" t="inlineStr"/>
-      <c r="AE39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8232,28 +6830,9 @@
       <c r="K40" t="n">
         <v>1</v>
       </c>
-      <c r="L40" t="inlineStr"/>
       <c r="M40" t="n">
         <v>1</v>
       </c>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr"/>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr"/>
-      <c r="X40" t="inlineStr"/>
-      <c r="Y40" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
-      <c r="AA40" t="inlineStr"/>
-      <c r="AB40" t="inlineStr"/>
-      <c r="AC40" t="inlineStr"/>
-      <c r="AD40" t="inlineStr"/>
-      <c r="AE40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8293,30 +6872,9 @@
       <c r="I41" t="n">
         <v>2</v>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
         <v>1</v>
       </c>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
-      <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
-      <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="inlineStr"/>
-      <c r="AA41" t="inlineStr"/>
-      <c r="AB41" t="inlineStr"/>
-      <c r="AC41" t="inlineStr"/>
-      <c r="AD41" t="inlineStr"/>
-      <c r="AE41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -8348,34 +6906,12 @@
       <c r="G42" t="n">
         <v>34</v>
       </c>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="n">
         <v>1</v>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" t="n">
         <v>1</v>
       </c>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
-      <c r="T42" t="inlineStr"/>
-      <c r="U42" t="inlineStr"/>
-      <c r="V42" t="inlineStr"/>
-      <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
-      <c r="Y42" t="inlineStr"/>
-      <c r="Z42" t="inlineStr"/>
-      <c r="AA42" t="inlineStr"/>
-      <c r="AB42" t="inlineStr"/>
-      <c r="AC42" t="inlineStr"/>
-      <c r="AD42" t="inlineStr"/>
-      <c r="AE42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -8415,30 +6951,9 @@
       <c r="I43" t="n">
         <v>3</v>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
       <c r="M43" t="n">
         <v>1</v>
       </c>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
-      <c r="T43" t="inlineStr"/>
-      <c r="U43" t="inlineStr"/>
-      <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr"/>
-      <c r="X43" t="inlineStr"/>
-      <c r="Y43" t="inlineStr"/>
-      <c r="Z43" t="inlineStr"/>
-      <c r="AA43" t="inlineStr"/>
-      <c r="AB43" t="inlineStr"/>
-      <c r="AC43" t="inlineStr"/>
-      <c r="AD43" t="inlineStr"/>
-      <c r="AE43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8478,30 +6993,9 @@
       <c r="I44" t="n">
         <v>1</v>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="n">
         <v>1</v>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
-      <c r="T44" t="inlineStr"/>
-      <c r="U44" t="inlineStr"/>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr"/>
-      <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr"/>
-      <c r="Z44" t="inlineStr"/>
-      <c r="AA44" t="inlineStr"/>
-      <c r="AB44" t="inlineStr"/>
-      <c r="AC44" t="inlineStr"/>
-      <c r="AD44" t="inlineStr"/>
-      <c r="AE44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -8533,34 +7027,12 @@
       <c r="G45" t="n">
         <v>34</v>
       </c>
-      <c r="H45" t="inlineStr"/>
       <c r="I45" t="n">
         <v>1</v>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
       <c r="O45" t="n">
         <v>1</v>
       </c>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
-      <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
-      <c r="Y45" t="inlineStr"/>
-      <c r="Z45" t="inlineStr"/>
-      <c r="AA45" t="inlineStr"/>
-      <c r="AB45" t="inlineStr"/>
-      <c r="AC45" t="inlineStr"/>
-      <c r="AD45" t="inlineStr"/>
-      <c r="AE45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8603,27 +7075,6 @@
       <c r="J46" t="n">
         <v>1</v>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
-      <c r="T46" t="inlineStr"/>
-      <c r="U46" t="inlineStr"/>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
-      <c r="Y46" t="inlineStr"/>
-      <c r="Z46" t="inlineStr"/>
-      <c r="AA46" t="inlineStr"/>
-      <c r="AB46" t="inlineStr"/>
-      <c r="AC46" t="inlineStr"/>
-      <c r="AD46" t="inlineStr"/>
-      <c r="AE46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8655,34 +7106,12 @@
       <c r="G47" t="n">
         <v>51</v>
       </c>
-      <c r="H47" t="inlineStr"/>
       <c r="I47" t="n">
         <v>4</v>
       </c>
       <c r="J47" t="n">
         <v>1</v>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr"/>
-      <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
-      <c r="Y47" t="inlineStr"/>
-      <c r="Z47" t="inlineStr"/>
-      <c r="AA47" t="inlineStr"/>
-      <c r="AB47" t="inlineStr"/>
-      <c r="AC47" t="inlineStr"/>
-      <c r="AD47" t="inlineStr"/>
-      <c r="AE47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8714,34 +7143,12 @@
       <c r="G48" t="n">
         <v>51</v>
       </c>
-      <c r="H48" t="inlineStr"/>
       <c r="I48" t="n">
         <v>5</v>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" t="n">
         <v>1</v>
       </c>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr"/>
-      <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
-      <c r="Y48" t="inlineStr"/>
-      <c r="Z48" t="inlineStr"/>
-      <c r="AA48" t="inlineStr"/>
-      <c r="AB48" t="inlineStr"/>
-      <c r="AC48" t="inlineStr"/>
-      <c r="AD48" t="inlineStr"/>
-      <c r="AE48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8778,31 +7185,9 @@
           <t>+1 a los Bonos máximos.</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
         <v>1</v>
       </c>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
-      <c r="T49" t="inlineStr"/>
-      <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
-      <c r="Y49" t="inlineStr"/>
-      <c r="Z49" t="inlineStr"/>
-      <c r="AA49" t="inlineStr"/>
-      <c r="AB49" t="inlineStr"/>
-      <c r="AC49" t="inlineStr"/>
-      <c r="AD49" t="inlineStr"/>
-      <c r="AE49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8842,30 +7227,9 @@
       <c r="I50" t="n">
         <v>1</v>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
-      <c r="T50" t="inlineStr"/>
-      <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr"/>
       <c r="X50" t="n">
         <v>1</v>
       </c>
-      <c r="Y50" t="inlineStr"/>
-      <c r="Z50" t="inlineStr"/>
-      <c r="AA50" t="inlineStr"/>
-      <c r="AB50" t="inlineStr"/>
-      <c r="AC50" t="inlineStr"/>
-      <c r="AD50" t="inlineStr"/>
-      <c r="AE50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8905,30 +7269,9 @@
       <c r="I51" t="n">
         <v>1</v>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
-      <c r="T51" t="inlineStr"/>
-      <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr"/>
       <c r="W51" t="n">
         <v>2</v>
       </c>
-      <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
-      <c r="Z51" t="inlineStr"/>
-      <c r="AA51" t="inlineStr"/>
-      <c r="AB51" t="inlineStr"/>
-      <c r="AC51" t="inlineStr"/>
-      <c r="AD51" t="inlineStr"/>
-      <c r="AE51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8962,34 +7305,25 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Otorga regeneración de +3hp x mantenimiento (aplicar a mano).</t>
+          <t>Regenera 3 HP por turno mientras los tengas equipados.</t>
         </is>
       </c>
       <c r="I52" t="n">
         <v>4</v>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
-      <c r="T52" t="inlineStr"/>
-      <c r="U52" t="inlineStr"/>
-      <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr"/>
-      <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr"/>
-      <c r="Z52" t="inlineStr"/>
-      <c r="AA52" t="inlineStr"/>
-      <c r="AB52" t="inlineStr"/>
-      <c r="AC52" t="inlineStr"/>
-      <c r="AD52" t="inlineStr"/>
-      <c r="AE52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>Regeneración (troll)</t>
+        </is>
+      </c>
+      <c r="AE52" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>La piel de troll regenera 3 HP en cada mantenimiento, mientras tengas los guantes puestos.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9029,30 +7363,9 @@
       <c r="I53" t="n">
         <v>1</v>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
-      <c r="T53" t="inlineStr"/>
-      <c r="U53" t="inlineStr"/>
-      <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
-      <c r="X53" t="inlineStr"/>
-      <c r="Y53" t="inlineStr"/>
-      <c r="Z53" t="inlineStr"/>
-      <c r="AA53" t="inlineStr"/>
-      <c r="AB53" t="inlineStr"/>
       <c r="AC53" t="n">
         <v>1</v>
       </c>
-      <c r="AD53" t="inlineStr"/>
-      <c r="AE53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9107,23 +7420,6 @@
       <c r="N54" t="n">
         <v>2</v>
       </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
-      <c r="T54" t="inlineStr"/>
-      <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
-      <c r="X54" t="inlineStr"/>
-      <c r="Y54" t="inlineStr"/>
-      <c r="Z54" t="inlineStr"/>
-      <c r="AA54" t="inlineStr"/>
-      <c r="AB54" t="inlineStr"/>
-      <c r="AC54" t="inlineStr"/>
-      <c r="AD54" t="inlineStr"/>
-      <c r="AE54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9178,25 +7474,9 @@
       <c r="N55" t="n">
         <v>1</v>
       </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
-      <c r="T55" t="inlineStr"/>
-      <c r="U55" t="inlineStr"/>
-      <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr"/>
-      <c r="X55" t="inlineStr"/>
-      <c r="Y55" t="inlineStr"/>
       <c r="Z55" t="n">
         <v>5</v>
       </c>
-      <c r="AA55" t="inlineStr"/>
-      <c r="AB55" t="inlineStr"/>
-      <c r="AC55" t="inlineStr"/>
-      <c r="AD55" t="inlineStr"/>
-      <c r="AE55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9228,38 +7508,18 @@
       <c r="G56" t="n">
         <v>338</v>
       </c>
-      <c r="H56" t="inlineStr"/>
       <c r="I56" t="n">
         <v>10</v>
       </c>
-      <c r="J56" t="inlineStr"/>
       <c r="K56" t="n">
         <v>1</v>
       </c>
-      <c r="L56" t="inlineStr"/>
       <c r="M56" t="n">
         <v>1</v>
       </c>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
-      <c r="T56" t="inlineStr"/>
-      <c r="U56" t="inlineStr"/>
       <c r="V56" t="n">
         <v>1</v>
       </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
-      <c r="Y56" t="inlineStr"/>
-      <c r="Z56" t="inlineStr"/>
-      <c r="AA56" t="inlineStr"/>
-      <c r="AB56" t="inlineStr"/>
-      <c r="AC56" t="inlineStr"/>
-      <c r="AD56" t="inlineStr"/>
-      <c r="AE56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -9291,36 +7551,15 @@
       <c r="G57" t="n">
         <v>186</v>
       </c>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="n">
         <v>6</v>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
         <v>2</v>
       </c>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57" t="n">
         <v>1</v>
       </c>
-      <c r="S57" t="inlineStr"/>
-      <c r="T57" t="inlineStr"/>
-      <c r="U57" t="inlineStr"/>
-      <c r="V57" t="inlineStr"/>
-      <c r="W57" t="inlineStr"/>
-      <c r="X57" t="inlineStr"/>
-      <c r="Y57" t="inlineStr"/>
-      <c r="Z57" t="inlineStr"/>
-      <c r="AA57" t="inlineStr"/>
-      <c r="AB57" t="inlineStr"/>
-      <c r="AC57" t="inlineStr"/>
-      <c r="AD57" t="inlineStr"/>
-      <c r="AE57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -9352,36 +7591,15 @@
       <c r="G58" t="n">
         <v>157</v>
       </c>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="n">
         <v>5</v>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
       <c r="M58" t="n">
         <v>1</v>
       </c>
-      <c r="N58" t="inlineStr"/>
       <c r="O58" t="n">
         <v>2</v>
       </c>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
-      <c r="T58" t="inlineStr"/>
-      <c r="U58" t="inlineStr"/>
-      <c r="V58" t="inlineStr"/>
-      <c r="W58" t="inlineStr"/>
-      <c r="X58" t="inlineStr"/>
-      <c r="Y58" t="inlineStr"/>
-      <c r="Z58" t="inlineStr"/>
-      <c r="AA58" t="inlineStr"/>
-      <c r="AB58" t="inlineStr"/>
-      <c r="AC58" t="inlineStr"/>
-      <c r="AD58" t="inlineStr"/>
-      <c r="AE58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -9424,29 +7642,9 @@
       <c r="J59" t="n">
         <v>1</v>
       </c>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
       <c r="Q59" t="n">
         <v>1</v>
       </c>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
-      <c r="T59" t="inlineStr"/>
-      <c r="U59" t="inlineStr"/>
-      <c r="V59" t="inlineStr"/>
-      <c r="W59" t="inlineStr"/>
-      <c r="X59" t="inlineStr"/>
-      <c r="Y59" t="inlineStr"/>
-      <c r="Z59" t="inlineStr"/>
-      <c r="AA59" t="inlineStr"/>
-      <c r="AB59" t="inlineStr"/>
-      <c r="AC59" t="inlineStr"/>
-      <c r="AD59" t="inlineStr"/>
-      <c r="AE59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -9501,23 +7699,6 @@
       <c r="N60" t="n">
         <v>1</v>
       </c>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
-      <c r="T60" t="inlineStr"/>
-      <c r="U60" t="inlineStr"/>
-      <c r="V60" t="inlineStr"/>
-      <c r="W60" t="inlineStr"/>
-      <c r="X60" t="inlineStr"/>
-      <c r="Y60" t="inlineStr"/>
-      <c r="Z60" t="inlineStr"/>
-      <c r="AA60" t="inlineStr"/>
-      <c r="AB60" t="inlineStr"/>
-      <c r="AC60" t="inlineStr"/>
-      <c r="AD60" t="inlineStr"/>
-      <c r="AE60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9563,26 +7744,6 @@
       <c r="K61" t="n">
         <v>1</v>
       </c>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
-      <c r="T61" t="inlineStr"/>
-      <c r="U61" t="inlineStr"/>
-      <c r="V61" t="inlineStr"/>
-      <c r="W61" t="inlineStr"/>
-      <c r="X61" t="inlineStr"/>
-      <c r="Y61" t="inlineStr"/>
-      <c r="Z61" t="inlineStr"/>
-      <c r="AA61" t="inlineStr"/>
-      <c r="AB61" t="inlineStr"/>
-      <c r="AC61" t="inlineStr"/>
-      <c r="AD61" t="inlineStr"/>
-      <c r="AE61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -9634,24 +7795,6 @@
       <c r="M62" t="n">
         <v>1</v>
       </c>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
-      <c r="T62" t="inlineStr"/>
-      <c r="U62" t="inlineStr"/>
-      <c r="V62" t="inlineStr"/>
-      <c r="W62" t="inlineStr"/>
-      <c r="X62" t="inlineStr"/>
-      <c r="Y62" t="inlineStr"/>
-      <c r="Z62" t="inlineStr"/>
-      <c r="AA62" t="inlineStr"/>
-      <c r="AB62" t="inlineStr"/>
-      <c r="AC62" t="inlineStr"/>
-      <c r="AD62" t="inlineStr"/>
-      <c r="AE62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -9703,24 +7846,6 @@
       <c r="M63" t="n">
         <v>1</v>
       </c>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
-      <c r="T63" t="inlineStr"/>
-      <c r="U63" t="inlineStr"/>
-      <c r="V63" t="inlineStr"/>
-      <c r="W63" t="inlineStr"/>
-      <c r="X63" t="inlineStr"/>
-      <c r="Y63" t="inlineStr"/>
-      <c r="Z63" t="inlineStr"/>
-      <c r="AA63" t="inlineStr"/>
-      <c r="AB63" t="inlineStr"/>
-      <c r="AC63" t="inlineStr"/>
-      <c r="AD63" t="inlineStr"/>
-      <c r="AE63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -9752,38 +7877,18 @@
       <c r="G64" t="n">
         <v>205</v>
       </c>
-      <c r="H64" t="inlineStr"/>
       <c r="I64" t="n">
         <v>9</v>
       </c>
       <c r="J64" t="n">
         <v>1</v>
       </c>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
       <c r="M64" t="n">
         <v>1</v>
       </c>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr"/>
       <c r="T64" t="n">
         <v>1</v>
       </c>
-      <c r="U64" t="inlineStr"/>
-      <c r="V64" t="inlineStr"/>
-      <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
-      <c r="Y64" t="inlineStr"/>
-      <c r="Z64" t="inlineStr"/>
-      <c r="AA64" t="inlineStr"/>
-      <c r="AB64" t="inlineStr"/>
-      <c r="AC64" t="inlineStr"/>
-      <c r="AD64" t="inlineStr"/>
-      <c r="AE64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9835,26 +7940,9 @@
       <c r="M65" t="n">
         <v>1</v>
       </c>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr"/>
       <c r="S65" t="n">
         <v>1</v>
       </c>
-      <c r="T65" t="inlineStr"/>
-      <c r="U65" t="inlineStr"/>
-      <c r="V65" t="inlineStr"/>
-      <c r="W65" t="inlineStr"/>
-      <c r="X65" t="inlineStr"/>
-      <c r="Y65" t="inlineStr"/>
-      <c r="Z65" t="inlineStr"/>
-      <c r="AA65" t="inlineStr"/>
-      <c r="AB65" t="inlineStr"/>
-      <c r="AC65" t="inlineStr"/>
-      <c r="AD65" t="inlineStr"/>
-      <c r="AE65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -9909,25 +7997,9 @@
       <c r="N66" t="n">
         <v>1</v>
       </c>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="inlineStr"/>
-      <c r="S66" t="inlineStr"/>
-      <c r="T66" t="inlineStr"/>
       <c r="U66" t="n">
         <v>1</v>
       </c>
-      <c r="V66" t="inlineStr"/>
-      <c r="W66" t="inlineStr"/>
-      <c r="X66" t="inlineStr"/>
-      <c r="Y66" t="inlineStr"/>
-      <c r="Z66" t="inlineStr"/>
-      <c r="AA66" t="inlineStr"/>
-      <c r="AB66" t="inlineStr"/>
-      <c r="AC66" t="inlineStr"/>
-      <c r="AD66" t="inlineStr"/>
-      <c r="AE66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -9967,30 +8039,9 @@
       <c r="I67" t="n">
         <v>2</v>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
       <c r="T67" t="n">
         <v>2</v>
       </c>
-      <c r="U67" t="inlineStr"/>
-      <c r="V67" t="inlineStr"/>
-      <c r="W67" t="inlineStr"/>
-      <c r="X67" t="inlineStr"/>
-      <c r="Y67" t="inlineStr"/>
-      <c r="Z67" t="inlineStr"/>
-      <c r="AA67" t="inlineStr"/>
-      <c r="AB67" t="inlineStr"/>
-      <c r="AC67" t="inlineStr"/>
-      <c r="AD67" t="inlineStr"/>
-      <c r="AE67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -10030,30 +8081,9 @@
       <c r="I68" t="n">
         <v>4</v>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
       <c r="P68" t="n">
         <v>1</v>
       </c>
-      <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
-      <c r="T68" t="inlineStr"/>
-      <c r="U68" t="inlineStr"/>
-      <c r="V68" t="inlineStr"/>
-      <c r="W68" t="inlineStr"/>
-      <c r="X68" t="inlineStr"/>
-      <c r="Y68" t="inlineStr"/>
-      <c r="Z68" t="inlineStr"/>
-      <c r="AA68" t="inlineStr"/>
-      <c r="AB68" t="inlineStr"/>
-      <c r="AC68" t="inlineStr"/>
-      <c r="AD68" t="inlineStr"/>
-      <c r="AE68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -10093,28 +8123,6 @@
       <c r="I69" t="n">
         <v>1</v>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
-      <c r="T69" t="inlineStr"/>
-      <c r="U69" t="inlineStr"/>
-      <c r="V69" t="inlineStr"/>
-      <c r="W69" t="inlineStr"/>
-      <c r="X69" t="inlineStr"/>
-      <c r="Y69" t="inlineStr"/>
-      <c r="Z69" t="inlineStr"/>
-      <c r="AA69" t="inlineStr"/>
-      <c r="AB69" t="inlineStr"/>
-      <c r="AC69" t="inlineStr"/>
-      <c r="AD69" t="inlineStr"/>
-      <c r="AE69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -10154,7 +8162,6 @@
       <c r="I70" t="n">
         <v>6</v>
       </c>
-      <c r="J70" t="inlineStr"/>
       <c r="K70" t="n">
         <v>1</v>
       </c>
@@ -10164,24 +8171,6 @@
       <c r="M70" t="n">
         <v>1</v>
       </c>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
-      <c r="T70" t="inlineStr"/>
-      <c r="U70" t="inlineStr"/>
-      <c r="V70" t="inlineStr"/>
-      <c r="W70" t="inlineStr"/>
-      <c r="X70" t="inlineStr"/>
-      <c r="Y70" t="inlineStr"/>
-      <c r="Z70" t="inlineStr"/>
-      <c r="AA70" t="inlineStr"/>
-      <c r="AB70" t="inlineStr"/>
-      <c r="AC70" t="inlineStr"/>
-      <c r="AD70" t="inlineStr"/>
-      <c r="AE70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10213,38 +8202,18 @@
       <c r="G71" t="n">
         <v>188</v>
       </c>
-      <c r="H71" t="inlineStr"/>
       <c r="I71" t="n">
         <v>8</v>
       </c>
       <c r="J71" t="n">
         <v>1</v>
       </c>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
       <c r="M71" t="n">
         <v>1</v>
       </c>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr"/>
       <c r="Q71" t="n">
         <v>1</v>
       </c>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
-      <c r="T71" t="inlineStr"/>
-      <c r="U71" t="inlineStr"/>
-      <c r="V71" t="inlineStr"/>
-      <c r="W71" t="inlineStr"/>
-      <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr"/>
-      <c r="Z71" t="inlineStr"/>
-      <c r="AA71" t="inlineStr"/>
-      <c r="AB71" t="inlineStr"/>
-      <c r="AC71" t="inlineStr"/>
-      <c r="AD71" t="inlineStr"/>
-      <c r="AE71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -10284,8 +8253,6 @@
       <c r="I72" t="n">
         <v>4</v>
       </c>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
       <c r="L72" t="n">
         <v>2</v>
       </c>
@@ -10295,23 +8262,6 @@
       <c r="N72" t="n">
         <v>1</v>
       </c>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
-      <c r="T72" t="inlineStr"/>
-      <c r="U72" t="inlineStr"/>
-      <c r="V72" t="inlineStr"/>
-      <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr"/>
-      <c r="Z72" t="inlineStr"/>
-      <c r="AA72" t="inlineStr"/>
-      <c r="AB72" t="inlineStr"/>
-      <c r="AC72" t="inlineStr"/>
-      <c r="AD72" t="inlineStr"/>
-      <c r="AE72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -10343,41 +8293,21 @@
       <c r="G73" t="n">
         <v>205</v>
       </c>
-      <c r="H73" t="inlineStr"/>
       <c r="I73" t="n">
         <v>9</v>
       </c>
-      <c r="J73" t="inlineStr"/>
       <c r="K73" t="n">
         <v>1</v>
       </c>
       <c r="L73" t="n">
         <v>1</v>
       </c>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="inlineStr"/>
       <c r="R73" t="n">
         <v>1</v>
       </c>
-      <c r="S73" t="inlineStr"/>
-      <c r="T73" t="inlineStr"/>
-      <c r="U73" t="inlineStr"/>
-      <c r="V73" t="inlineStr"/>
-      <c r="W73" t="inlineStr"/>
-      <c r="X73" t="inlineStr"/>
-      <c r="Y73" t="inlineStr"/>
-      <c r="Z73" t="inlineStr"/>
-      <c r="AA73" t="inlineStr"/>
-      <c r="AB73" t="inlineStr"/>
-      <c r="AC73" t="inlineStr"/>
-      <c r="AD73" t="inlineStr"/>
-      <c r="AE73" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE73"/>
+  <autoFilter ref="A1:AH73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Estados nuevos, catálogo a 309 ítems, GM con catálogo completo y dock con color
- Presets "Rompe armadura" (mitad de Defensa/Res.crít total), "Arruina
  armadura" (anula solo el aporte del slot armadura, no todo el equipo),
  "Veneno severo" (daño creciente, no caduca) y "Sangrado" (-2 HP/turno,
  permanente) en ficha.html y gm-tools.html.
- Importada la actualización del Excel: 265 -> 309 ítems, Excel
  regenerado con los IDs nuevos, imágenes de "Poción de Bonos" cargadas.
- GM tools: el catálogo completo ahora incluye consumibles (solo lectura,
  no equipables), y nuevo botón "Ítem custom" para crear equipo desde
  cero y equiparlo directo a un creep.
- Ficha: botones del dock con tonalidades y emoji propios para
  identificarlos de un vistazo.
- Catálogos del fabricante (ficha y GM): el orden por defecto pasa a ser
  por tier ascendente (Común -> Legendario) dentro de cada categoría.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Consumibles'!$A$1:$T$130</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$U$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$U$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Escudos'!$A$1:$U$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defensivos'!$A$1:$AH$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Otros'!$A$1:$Q$2</definedName>
@@ -674,7 +674,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
         <v>30</v>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Otorga +1 a HP máximo durante todo el combate. Al usarlo se activa el estado 'Vitalidad Extendida (pergamino)'.</t>
+          <t>Otorga +10 a HP máximo durante todo el combate. Al usarlo se activa el estado 'Vitalidad Extendida (pergamino)'.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>HP máximo +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
+          <t>HP máximo +10. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Otorga +2 a HP máximo durante 4 turnos. Al consumirla se activa el estado 'Vitalidad Extendida mayor (poción)'.</t>
+          <t>Otorga +20 a HP máximo durante 4 turnos. Al consumirla se activa el estado 'Vitalidad Extendida mayor (poción)'.</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -3303,7 +3303,7 @@
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>HP máximo +2 mientras dure (4 turnos).</t>
+          <t>HP máximo +20 mientras dure (4 turnos).</t>
         </is>
       </c>
       <c r="S45" t="inlineStr"/>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Otorga +1 a HP máximo durante 4 turnos. Al consumirla se activa el estado 'Vitalidad Extendida (poción)'.</t>
+          <t>Otorga +10 a HP máximo durante 4 turnos. Al consumirla se activa el estado 'Vitalidad Extendida (poción)'.</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -4601,7 +4601,7 @@
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr">
         <is>
-          <t>HP máximo +1 mientras dure (4 turnos).</t>
+          <t>HP máximo +10 mientras dure (4 turnos).</t>
         </is>
       </c>
       <c r="S66" t="inlineStr"/>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Otorga +3 a HP máximo durante todo el combate. Al usarlo se activa el estado 'Vitalidad Extendida superior (pergamino)'.</t>
+          <t>Otorga +30 a HP máximo durante todo el combate. Al usarlo se activa el estado 'Vitalidad Extendida superior (pergamino)'.</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -5669,7 +5669,7 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>HP máximo +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
+          <t>HP máximo +30. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
       <c r="S83" t="inlineStr"/>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Otorga +2 a HP máximo durante todo el combate. Al usarlo se activa el estado 'Vitalidad Extendida mayor (pergamino)'.</t>
+          <t>Otorga +20 a HP máximo durante todo el combate. Al usarlo se activa el estado 'Vitalidad Extendida mayor (pergamino)'.</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -7017,7 +7017,7 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>HP máximo +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
+          <t>HP máximo +20. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
       <c r="S105" t="inlineStr"/>
@@ -8379,7 +8379,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Otorga +3 a HP máximo durante 4 turnos. Al consumirla se activa el estado 'Vitalidad Extendida superior (poción)'.</t>
+          <t>Otorga +30 a HP máximo durante 4 turnos. Al consumirla se activa el estado 'Vitalidad Extendida superior (poción)'.</t>
         </is>
       </c>
       <c r="I128" t="inlineStr"/>
@@ -8403,7 +8403,7 @@
       <c r="Q128" t="inlineStr"/>
       <c r="R128" t="inlineStr">
         <is>
-          <t>HP máximo +3 mientras dure (4 turnos).</t>
+          <t>HP máximo +30 mientras dure (4 turnos).</t>
         </is>
       </c>
       <c r="S128" t="inlineStr"/>
@@ -8555,7 +8555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8691,12 +8691,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>new-daga-de-capitan</t>
+          <t>new-baculo-de-batalla</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Daga de Capitán</t>
+          <t>Báculo de batalla</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8710,28 +8710,26 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>pdg +1</t>
+          <t>rango +1, bloqueo +1</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -8746,12 +8744,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>new-daga-de-guardia</t>
+          <t>new-cimitarra-de-guardia</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Daga de guardia</t>
+          <t>Cimitarra de guardia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8771,23 +8769,25 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Ignora 1 punto de resistencia al crítico</t>
+          <t>Parry +2</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>2</v>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
@@ -8799,12 +8799,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cat-espada-ancha</t>
+          <t>new-daga-de-capitan</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Espada ancha</t>
+          <t>Daga de Capitán</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -8821,23 +8821,25 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Daño amplificado.</t>
+          <t>pdg +1</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -8847,21 +8849,17 @@
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cat-espada-larga</t>
+          <t>new-daga-de-guardia</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Espada larga</t>
+          <t>Daga de guardia</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -8875,28 +8873,26 @@
         </is>
       </c>
       <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>60</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Ignora 1 punto de resistencia al crítico</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>80</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Pdg +1</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>4</v>
-      </c>
       <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
@@ -8906,21 +8902,17 @@
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>new-estilete-de-competencia</t>
+          <t>cat-espada-larga</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Estilete de competencia</t>
+          <t>Espada larga</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -8934,26 +8926,28 @@
         </is>
       </c>
       <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>90</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>pdg +2</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>75</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Crítico +1</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -8963,17 +8957,21 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cat-estoque</t>
+          <t>new-estilete-de-competencia</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Estoque</t>
+          <t>Estilete de competencia</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -8990,14 +8988,14 @@
         <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Modificador: +1 a iniciativa</t>
+          <t>Crítico +1</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -9008,9 +9006,7 @@
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" t="n">
-        <v>1</v>
-      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
@@ -9018,21 +9014,17 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cat-hacha-de-batalla</t>
+          <t>cat-estoque</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hacha de batalla</t>
+          <t>Estoque</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -9052,27 +9044,27 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Rompe armadura. +1 al bloqueo</t>
+          <t>Modificador: +1 a iniciativa</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="n">
-        <v>1</v>
-      </c>
+      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
@@ -9086,12 +9078,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>new-hacha-de-guerra-ligera</t>
+          <t>new-falchion</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hacha de guerra ligera</t>
+          <t>Falchion</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -9105,24 +9097,24 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Rompe armadura</t>
+          <t>Ingora 1 de resistencia al crítico</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
@@ -9139,12 +9131,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cat-martillo</t>
+          <t>new-hacha-con-pico</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Martillo</t>
+          <t>Hacha con pico</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -9158,24 +9150,24 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Daño +50%. Lento.</t>
+          <t>ignora 1 de resistencia al crítico</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
@@ -9187,21 +9179,17 @@
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>new-martillo-de-sargento</t>
+          <t>cat-hacha-de-batalla</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Martillo de sargento</t>
+          <t>Hacha de batalla</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -9215,50 +9203,52 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Tipo de daño: Tipo 8 (Impacto/contundente).</t>
+          <t>Rompe armadura. +1 al bloqueo</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="n">
-        <v>10</v>
-      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
-        <v>1</v>
-      </c>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>new-pico-de-guerra</t>
+          <t>new-hacha-de-doble-filo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pico de guerra</t>
+          <t>Hacha de doble filo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -9272,24 +9262,24 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>rango +1, 50% de romper armadura</t>
+          <t>Rompe armadura.</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
@@ -9306,12 +9296,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cat-rompemalla</t>
+          <t>new-hacha-de-guerra-ligera</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Rompemalla</t>
+          <t>Hacha de guerra ligera</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9331,18 +9321,14 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>75</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>50% chance de Romper armadura.</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -9354,21 +9340,17 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>new-sable-de-caballeria</t>
+          <t>new-hacha-dentada</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sable de caballería</t>
+          <t>Hacha dentada</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -9388,18 +9370,20 @@
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>87</v>
-      </c>
-      <c r="H14" t="inlineStr"/>
+        <v>115</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>50% de dejar sangrando</t>
+        </is>
+      </c>
       <c r="I14" t="n">
         <v>6</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
@@ -9414,17 +9398,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>new-cachiporra</t>
+          <t>cat-martillo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cachiporra</t>
+          <t>Martillo</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -9433,19 +9417,15 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>40</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Tipo de daño: Tipo 8 (Impacto/contundente).</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
         <v>8</v>
       </c>
@@ -9453,9 +9433,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="n">
-        <v>10</v>
-      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
@@ -9464,22 +9442,26 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>new-cimitarra</t>
+          <t>new-martillo-de-cabeza-plana</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cimitarra</t>
+          <t>Martillo de cabeza plana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -9488,21 +9470,21 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>55</v>
+        <v>135</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>parry +1</t>
+          <t>bloqueo +2</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -9510,9 +9492,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
@@ -9524,17 +9504,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>new-cuchillo-de-cazador</t>
+          <t>new-martillo-ergonomico</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cuchillo de cazador</t>
+          <t>Martillo ergonómico</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -9546,14 +9526,18 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>30</v>
-      </c>
-      <c r="H17" t="inlineStr"/>
+        <v>130</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>bloqueo +3</t>
+        </is>
+      </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -9573,17 +9557,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>new-daga</t>
+          <t>new-maza-de-guardia</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Daga</t>
+          <t>Maza de guardia</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -9592,20 +9576,20 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -9622,17 +9606,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cat-espada-corta</t>
+          <t>new-pico-de-guerra</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Espada corta</t>
+          <t>Pico de guerra</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -9641,17 +9625,21 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>30</v>
-      </c>
-      <c r="H19" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>rango +1, 50% de romper armadura</t>
+        </is>
+      </c>
       <c r="I19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -9666,26 +9654,22 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>new-espada-corta-de-instruccion</t>
+          <t>new-sable-de-caballeria</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Espada corta de instrucción</t>
+          <t>Sable de caballería</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -9694,25 +9678,33 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>50</v>
-      </c>
-      <c r="H20" t="inlineStr"/>
+        <v>75</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>pdg +1, parry +1</t>
+        </is>
+      </c>
       <c r="I20" t="n">
         <v>4</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
@@ -9724,17 +9716,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>new-estileto-comun</t>
+          <t>new-sable-militar</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Estileto común</t>
+          <t>Sable militar</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Común</t>
+          <t>Buena Calidad</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -9743,26 +9735,28 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>crítico +1</t>
+          <t>pdg +1</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
@@ -9777,12 +9771,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cat-hacha</t>
+          <t>new-baston-de-monje</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Hacha</t>
+          <t>Bastón de monje</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -9799,21 +9793,21 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Rompe armadura.</t>
+          <t>rango +1</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
@@ -9825,21 +9819,17 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>new-horquilla</t>
+          <t>new-bate-de-baseball</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Horquilla</t>
+          <t>Bate de Baseball</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -9859,18 +9849,14 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>50</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>rango +1</t>
-        </is>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
@@ -9887,12 +9873,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>new-hoz</t>
+          <t>new-cachiporra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Hoz</t>
+          <t>Cachiporra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -9909,20 +9895,22 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>10</v>
+      </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
@@ -9936,12 +9924,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>new-lanza-corta</t>
+          <t>new-cimitarra</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Lanza corta</t>
+          <t>Cimitarra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -9955,21 +9943,21 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>rango +1</t>
+          <t>parry +1</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -9977,7 +9965,9 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>1</v>
+      </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
@@ -9989,12 +9979,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>new-machete</t>
+          <t>new-cuchillo-de-cazador</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Machete</t>
+          <t>Cuchillo de cazador</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -10011,18 +10001,14 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>60</v>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>romper armadura 50%</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -10042,12 +10028,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>cat-maza</t>
+          <t>new-daga</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Maza</t>
+          <t>Daga</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -10061,21 +10047,17 @@
         </is>
       </c>
       <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>40</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="n">
         <v>2</v>
-      </c>
-      <c r="F27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" t="n">
-        <v>66</v>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Bloqueo +1</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>8</v>
       </c>
       <c r="J27" t="n">
         <v>1</v>
@@ -10090,21 +10072,17 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>new-maza-de-guardia</t>
+          <t>cat-espada-ancha</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Maza de guardia</t>
+          <t>Espada ancha</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -10118,24 +10096,20 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>55</v>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Bloqueo +1</t>
-        </is>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -10147,17 +10121,21 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>new-pica-hielos</t>
+          <t>cat-espada-corta</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pica Hielos</t>
+          <t>Espada corta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -10171,17 +10149,17 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -10196,17 +10174,21 @@
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>new-sable</t>
+          <t>new-espada-corta-de-instruccion</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sable</t>
+          <t>Espada corta de instrucción</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -10220,19 +10202,15 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>40</v>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>iniciativa +1</t>
-        </is>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="n">
         <v>4</v>
       </c>
@@ -10254,17 +10232,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>new-colmillo-dientes-de-sable</t>
+          <t>new-espada-corta-oxidada</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Colmillo dientes de sable</t>
+          <t>Espada corta oxidada</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -10273,24 +10251,24 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Deja sangrando x2hp</t>
+          <t>envenena x 50% de chances</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -10307,17 +10285,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>new-espadon</t>
+          <t>new-estileto-comun</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Espadón</t>
+          <t>Estileto común</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -10326,33 +10304,29 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>bloqueo +2</t>
+          <t>crítico +1</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="n">
-        <v>10</v>
-      </c>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="n">
-        <v>1</v>
-      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
@@ -10364,17 +10338,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>new-martillo-de-guerra-runico</t>
+          <t>cat-maza</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Martillo de guerra rúnico</t>
+          <t>Garrote</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -10383,53 +10357,51 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>170</v>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>25% de chances de dejar en pajaritos</t>
-        </is>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
         <v>8</v>
       </c>
       <c r="J33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
-      <c r="O33" t="n">
-        <v>1</v>
-      </c>
+      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
-      <c r="U33" t="inlineStr"/>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>new-punal-de-dorne</t>
+          <t>cat-hacha</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Puñal de Dorne</t>
+          <t>Hacha</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Excepcional</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -10438,24 +10410,24 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Veneno stock 4</t>
+          <t>Rompe armadura.</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -10467,22 +10439,26 @@
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>new-aguijon-de-manticora</t>
+          <t>new-hacha-de-constructor</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Aguijón de mantícora</t>
+          <t>Hacha de constructor</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Legendario</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -10491,21 +10467,21 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>500</v>
+        <v>90</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>critico +2, dza +2, 50% de chance de stunear</t>
+          <t>Rompe armadura</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -10525,17 +10501,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>new-aguijon-de-esgrima</t>
+          <t>new-hacha-de-lenador</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Aguijón de esgrima</t>
+          <t>Hacha de leñador</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -10550,15 +10526,11 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>110</v>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>parry +2, pdg +1</t>
-        </is>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -10578,17 +10550,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>new-espada-bastarda</t>
+          <t>new-hacha-oxidada</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Espada bastarda</t>
+          <t>Hacha oxidada</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -10597,21 +10569,21 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>parry+1, bloqueo+1</t>
+          <t>50% de chances de envenenar</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -10631,17 +10603,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>new-estoque-de-duelista</t>
+          <t>new-hachuela</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Estoque de duelista</t>
+          <t>Hachuela</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -10653,27 +10625,21 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>80</v>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Ingora 2 de resistencia al crítico</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="n">
-        <v>1</v>
-      </c>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
@@ -10686,17 +10652,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>cat-hacha-de-mano</t>
+          <t>new-horquilla</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Hacha de doble filo</t>
+          <t>Horquilla</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -10705,21 +10671,21 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Rompe armadura. Ignora 1 resistencia al crítico</t>
+          <t>rango +1</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -10734,26 +10700,22 @@
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>new-lanza-militar</t>
+          <t>new-hoz</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Lanza militar</t>
+          <t>Hoz</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -10762,24 +10724,24 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Daño amplificado.</t>
+          <t>sangrado 50%</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
@@ -10796,17 +10758,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>cat-mangual</t>
+          <t>new-lanza-corta</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Mangual</t>
+          <t>Lanza corta</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -10818,21 +10780,21 @@
         <v>2</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>120</v>
+        <v>75</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Alcance +1.</t>
+          <t>rango +1</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
@@ -10844,26 +10806,22 @@
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr"/>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="U41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>new-punal-aserrado</t>
+          <t>new-machete</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Puñal aserrado</t>
+          <t>Machete</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Raro</t>
+          <t>Común</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -10872,21 +10830,21 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Rompe armadura.</t>
+          <t>romper armadura 50%</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -10903,8 +10861,2376 @@
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>new-martillo-de-bola</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Martillo de bola</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>115</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>bloqueo +1</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>8</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>new-martillo-de-cantero</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Martillo de cantero</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>70</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>rango +1</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>8</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>new-maza-de-hierro</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Maza de hierro</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>90</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>bloqueo +1</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>8</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>new-pica-hielos</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Pica Hielos</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>40</v>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="n">
+        <v>2</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>new-sable-comun</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Sable común</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>40</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>iniciativa +1</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>4</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>new-tomahawk</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Tomahawk</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>60</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>rango +1</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>6</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>new-garrote-de-hueso</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>garrote de hueso</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Común</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>120</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>bloqueo +1</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>8</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>new-baculo-shao-lin</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Báculo Shao Lin</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
+        <v>800</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>parry+2, bloqueo +1, rango +1</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>8</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>new-colmillo-dientes-de-sable</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Colmillo dientes de sable</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>900</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Deja sangrando x2hp</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>2</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>new-espada-larga-de-dorne</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Espada larga de Dorne</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>500</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>pdg+2, envenena</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>4</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1</v>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>new-espadon</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Espadón</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>4</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="n">
+        <v>500</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>parry +2, bloqueo +3</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>4</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="n">
+        <v>10</v>
+      </c>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="n">
+        <v>1</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>new-flamberge</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Flamberge</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" t="n">
+        <v>550</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>sangrado, +1 pdg</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>4</v>
+      </c>
+      <c r="J54" t="n">
+        <v>2</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1</v>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>new-gladius</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Gladius</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>400</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>parry +2, bloqueo +2</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>4</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="n">
+        <v>2</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>new-hacha-de-guardia-real</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Hacha de guardia real</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>2</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
+        <v>500</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>parry +2, bloqueo +3</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>6</v>
+      </c>
+      <c r="J56" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>new-hacha-de-madera-mistica</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Hacha de madera mística</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>2</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>600</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Rompe armadura. Drena 50% del daño.</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>6</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr"/>
+      <c r="U57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>new-hacha-filo-de-diamante</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Hacha filo de diamante</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>3</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>450</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Crítico aumentado. Arruina armadura.</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>6</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>new-martillo-de-guerra-runico</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Martillo de guerra rúnico</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>3</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" t="n">
+        <v>850</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Deja en pajaritos</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>8</v>
+      </c>
+      <c r="J59" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="n">
+        <v>1</v>
+      </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>new-punal-de-dorne</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Puñal de Dorne</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
+        <v>850</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Veneno stock 4</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>2</v>
+      </c>
+      <c r="J60" t="n">
+        <v>2</v>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>new-rompefilas</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Rompefilas</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Excepcional</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>900</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Expulsa 2 casilleros para atrás + FUERZA vs CONST. Si choca contra algo, daño directo igual a la diferencia</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>8</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>new-aguijon-de-manticora</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Aguijón de mantícora</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>critico +2, dza +2, aplica veneno severo</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>2</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>new-espada-de-nosferatu</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Espada de Nosferatu</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1300</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>50% de chances de ignorar armadura. Drena hp igual al daño ejercido</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>new-garra-de-fafner</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Garra de Fafner</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Ignora armadura. Cada golpe consecutivo al mismo enemigo aumenta en 1 el daño fijo del hacha.</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>6</v>
+      </c>
+      <c r="J64" t="n">
+        <v>1</v>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr"/>
+      <c r="U64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>new-hacha-de-durin</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Hacha de Durin</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Arruina armadura. +2 a la fuerza. deja lisiado</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>6</v>
+      </c>
+      <c r="J65" t="n">
+        <v>1</v>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr"/>
+      <c r="U65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>new-martillo-de-vulcano</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Martillo de Vulcano</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>5</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="n">
+        <v>1600</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Hace daño explosivo en forma de cono de 3 hex detrás del objetivo golpeado</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>8</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr"/>
+      <c r="U66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>new-maza-de-vibranium</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Maza de vibranium</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>4</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>La mitad del daño ignora armadura. bloqueo +3</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>8</v>
+      </c>
+      <c r="J67" t="n">
+        <v>2</v>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>new-reflejo-de-acero</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Reflejo de Acero</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Legendario</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Parry +3, bloqueo +2, si bloquea con éxito, Gana derecho a un contraataque que no cuesta acciones</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>4</v>
+      </c>
+      <c r="J68" t="n">
+        <v>3</v>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>new-aguijon-de-esgrima</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Aguijón de esgrima</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>110</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>parry +2, pdg +1</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>2</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr"/>
+      <c r="U69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>new-cuchilla-de-carnicero</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Cuchilla de carnicero</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>110</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Rompe armadura</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>4</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>new-espada-bastarda</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Espada bastarda</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" t="n">
+        <v>120</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>parry+1, bloqueo+1</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>4</v>
+      </c>
+      <c r="J71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="n">
+        <v>1</v>
+      </c>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>new-estoque-de-duelista</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Estoque de duelista</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="n">
+        <v>80</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Ingora 2 de resistencia al crítico</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>2</v>
+      </c>
+      <c r="J72" t="n">
+        <v>2</v>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="n">
+        <v>1</v>
+      </c>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>new-hacha-danesa</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Hacha danesa</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>2</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" t="n">
+        <v>130</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Rango +1. Rompe armadura. Un hacha vikinga de asta larga y hoja delgada muy veloz y letal.</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>6</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
+      <c r="U73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>cat-hacha-de-mano</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Hacha de doble filo</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>3</v>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" t="n">
+        <v>120</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Rompe armadura. Ignora 1 resistencia al crítico</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>6</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>new-hacha-de-guerra-pesada</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Hacha de guerra pesada</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="n">
+        <v>130</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Arruina armadura</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>6</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>new-katana</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Katana</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" t="n">
+        <v>120</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>pdg+2, crítico +1</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>4</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
+        <v>2</v>
+      </c>
+      <c r="L76" t="n">
+        <v>1</v>
+      </c>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>new-lanza-militar</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Lanza militar</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>2</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" t="n">
+        <v>110</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>rango +1</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>2</v>
+      </c>
+      <c r="J77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
+      <c r="U77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>new-lucero-del-alba</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Lucero del alba</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="n">
+        <v>150</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Ignora 1 de res al crítico, rango +1</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>8</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
+      <c r="U78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>new-mandoble</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Mandoble</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>110</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Parry+2, bloqueo+1</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>4</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="n">
+        <v>2</v>
+      </c>
+      <c r="O79" t="inlineStr"/>
+      <c r="P79" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr"/>
+      <c r="U79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>cat-mangual</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Mangual</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" t="n">
+        <v>160</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Alcance +1.</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>8</v>
+      </c>
+      <c r="J80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr"/>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>new-mangual</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Mangual</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>4</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>150</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>rango +1</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>8</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr"/>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr"/>
+      <c r="U81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>new-martillo-de-sargento</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Martillo de sargento</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>4</v>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" t="n">
+        <v>140</v>
+      </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="n">
+        <v>8</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="n">
+        <v>10</v>
+      </c>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="n">
+        <v>1</v>
+      </c>
+      <c r="O82" t="inlineStr"/>
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr"/>
+      <c r="U82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>new-maza-de-acero</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Maza de acero</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>3</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
+        <v>160</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Bloqueo +3</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>8</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr"/>
+      <c r="U83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>new-punal-aserrado</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Puñal aserrado</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
+        <v>100</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Rompe armadura.</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>2</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="inlineStr"/>
+      <c r="U84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>cat-rompemalla</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Rompemalla</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" t="n">
+        <v>75</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>50% chance de Romper armadura.</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>2</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
+      <c r="P85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
+      <c r="T85" t="inlineStr"/>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>new-sagaris</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Sagaris</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>arma_1m</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" t="n">
+        <v>130</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Rompe armadura. Sangrado.</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>6</v>
+      </c>
+      <c r="J86" t="n">
+        <v>1</v>
+      </c>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
+      <c r="P86" t="inlineStr"/>
+      <c r="Q86" t="inlineStr"/>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr"/>
+      <c r="T86" t="inlineStr"/>
+      <c r="U86" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U42"/>
+  <autoFilter ref="A1:U86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11840,7 +14166,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>190</v>
+        <v>650</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -11891,7 +14217,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>220</v>
+        <v>750</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -11942,7 +14268,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>250</v>
+        <v>850</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -12009,11 +14335,11 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>600</v>
+        <v>1100</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>parry  +4, bloqueo +4, inmuniza ruptura de armadura</t>
+          <t>parry  +4, bloqueo +4, inmuniza rupturas de armadura</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -15644,14 +17970,16 @@
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>+1 a los Bonos máximos.</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="n">
+        <v>1</v>
+      </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
@@ -15708,7 +18036,7 @@
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>180</v>
+        <v>500</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -15774,7 +18102,7 @@
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>250</v>
+        <v>650</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -15840,7 +18168,7 @@
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -15970,7 +18298,7 @@
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -16044,7 +18372,7 @@
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -17700,7 +20028,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>41 ítems</t>
+          <t>85 ítems</t>
         </is>
       </c>
     </row>
@@ -17748,7 +20076,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>265 ítems</t>
+          <t>309 ítems</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catálogo: completar el modificador de Bloqueo que faltaba en 18 ítems
Varios items (mazas, martillos, báculos, escudos) mencionaban "bloqueo
+N" en el Detalle pero no tenían el modificador cargado, así que nunca
sumaba al stat secundario Bloqueo al equiparse. Se completó a mano en
el Excel, leyendo el valor del propio texto de Detalle, y se reimportó.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -8734,7 +8734,9 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
@@ -9494,7 +9496,9 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="n">
+        <v>2</v>
+      </c>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
@@ -9547,7 +9551,9 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="n">
+        <v>3</v>
+      </c>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
@@ -10907,7 +10913,9 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
+      <c r="P43" t="n">
+        <v>1</v>
+      </c>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
@@ -11013,7 +11021,9 @@
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
+      <c r="P45" t="n">
+        <v>1</v>
+      </c>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
@@ -11221,7 +11231,9 @@
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
+      <c r="P49" t="n">
+        <v>1</v>
+      </c>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
@@ -11274,7 +11286,9 @@
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
+      <c r="P50" t="n">
+        <v>1</v>
+      </c>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr"/>
@@ -11439,7 +11453,9 @@
         <v>1</v>
       </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
+      <c r="P53" t="n">
+        <v>3</v>
+      </c>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr"/>
       <c r="S53" t="inlineStr"/>
@@ -11604,7 +11620,9 @@
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
+      <c r="P56" t="n">
+        <v>3</v>
+      </c>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
@@ -12189,7 +12207,9 @@
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
+      <c r="P67" t="n">
+        <v>3</v>
+      </c>
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr"/>
       <c r="S67" t="inlineStr"/>
@@ -12242,7 +12262,9 @@
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
+      <c r="P68" t="n">
+        <v>2</v>
+      </c>
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
@@ -13059,7 +13081,9 @@
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" t="inlineStr"/>
+      <c r="P83" t="n">
+        <v>3</v>
+      </c>
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr"/>
       <c r="S83" t="inlineStr"/>
@@ -13695,7 +13719,11 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>bloqueo:2</t>
+        </is>
+      </c>
       <c r="U7" t="inlineStr">
         <is>
           <t>sí</t>
@@ -13807,7 +13835,11 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>bloqueo:2</t>
+        </is>
+      </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -14186,7 +14218,11 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>bloqueo:1</t>
+        </is>
+      </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -14237,7 +14273,11 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>bloqueo:1</t>
+        </is>
+      </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -14355,7 +14395,11 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>bloqueo:4</t>
+        </is>
+      </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -14581,7 +14625,11 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>bloqueo:2</t>
+        </is>
+      </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Renombrar Res.M (Int) a "Resistencia mental" / Res.Mt, sin tocar Res.Mg
Res.M y Res.Mg sonaban casi igual y se confundían. Res.M (derivado de
Inteligencia) pasa a llamarse Res.Mt / Resistencia mental en los tres
archivos (ficha, GM tools, vendor generator), en los dos ítems del
catálogo que la usan como modificador (Guantes de piel de unicornio,
Mercury threads) y en las herramientas de Excel (encabezado de columna).
Res.Mg (derivado de Constitución) queda exactamente igual.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -14954,7 +14954,7 @@
       </c>
       <c r="Z1" s="2" t="inlineStr">
         <is>
-          <t>Res. mágica</t>
+          <t>Res. mental</t>
         </is>
       </c>
       <c r="AA1" s="2" t="inlineStr">
@@ -15904,7 +15904,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>+1 a los Bonos máximos, +1 Res.M y +1 Res.CC.</t>
+          <t>+1 a los Bonos máximos, +1 Res.Mt y +1 Res.CC.</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -18516,7 +18516,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Resistencia a todos los críticos. +5 a resistencia mágica</t>
+          <t>Resistencia a todos los críticos. +5 a resistencia mental</t>
         </is>
       </c>
       <c r="I55" t="n">

</xml_diff>

<commit_message>
Catálogo: mecánica real para los pergaminos de stat plano
Misma familia de bug que las pociones: los 44 "Pergamino de X (mayor/
superior)" ya tenían Estado que aplica = "Nombre (pergamino)" y Estado
permanente tildado, pero Modificadores del estado vacío — usarlos
activaba un estado permanente que no hacía nada. Completé el modificador
parseando el propio Detalle de cada ítem, igual que con las pociones.
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -735,7 +735,11 @@
           <t>Resistencia mágica +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>resmg:1</t>
+        </is>
+      </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
     </row>
@@ -808,7 +812,11 @@
           <t>Rango de Casteo +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>rangocasteo:1</t>
+        </is>
+      </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
     </row>
@@ -881,7 +889,11 @@
           <t>Probabilidad de golpe mágico +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>pdgmg:1</t>
+        </is>
+      </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
     </row>
@@ -954,7 +966,11 @@
           <t>Daño +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>dmg:1</t>
+        </is>
+      </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
     </row>
@@ -1027,7 +1043,11 @@
           <t>Bloqueo +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>bloqueo:1</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
     </row>
@@ -1100,7 +1120,11 @@
           <t>Crítico +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>crit:1</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
     </row>
@@ -1173,7 +1197,11 @@
           <t>Evasión +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>eva:1</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
     </row>
@@ -1246,7 +1274,11 @@
           <t>Movimiento +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>mov:1</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
     </row>
@@ -1319,7 +1351,11 @@
           <t>Probabilidad de Golpe +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>pdg:1</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
     </row>
@@ -1392,7 +1428,11 @@
           <t>Rango +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>rng:1</t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
     </row>
@@ -1465,7 +1505,11 @@
           <t>Parry +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>parry:1</t>
+        </is>
+      </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
     </row>
@@ -1538,7 +1582,11 @@
           <t>Bonos máximos +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>bonos:1</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
     </row>
@@ -1611,7 +1659,11 @@
           <t>HP máximo +10. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>hpmax:10</t>
+        </is>
+      </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
     </row>
@@ -1684,7 +1736,11 @@
           <t>Resistencia a CC +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>rescc:1</t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
     </row>
@@ -2147,7 +2203,11 @@
           <t>Acciones máximas +1. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>accionesmax:1</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
     </row>
@@ -5599,7 +5659,11 @@
           <t>Resistencia mágica +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S71" t="inlineStr"/>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>resmg:3</t>
+        </is>
+      </c>
       <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr"/>
     </row>
@@ -5672,7 +5736,11 @@
           <t>Rango de Casteo +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S72" t="inlineStr"/>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>rangocasteo:3</t>
+        </is>
+      </c>
       <c r="T72" t="inlineStr"/>
       <c r="U72" t="inlineStr"/>
     </row>
@@ -5745,7 +5813,11 @@
           <t>Probabilidad de golpe mágico +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S73" t="inlineStr"/>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>pdgmg:3</t>
+        </is>
+      </c>
       <c r="T73" t="inlineStr"/>
       <c r="U73" t="inlineStr"/>
     </row>
@@ -5818,7 +5890,11 @@
           <t>Daño +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S74" t="inlineStr"/>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>dmg:3</t>
+        </is>
+      </c>
       <c r="T74" t="inlineStr"/>
       <c r="U74" t="inlineStr"/>
     </row>
@@ -5891,7 +5967,11 @@
           <t>Bloqueo +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S75" t="inlineStr"/>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>bloqueo:3</t>
+        </is>
+      </c>
       <c r="T75" t="inlineStr"/>
       <c r="U75" t="inlineStr"/>
     </row>
@@ -5964,7 +6044,11 @@
           <t>Crítico +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S76" t="inlineStr"/>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>crit:3</t>
+        </is>
+      </c>
       <c r="T76" t="inlineStr"/>
       <c r="U76" t="inlineStr"/>
     </row>
@@ -6037,7 +6121,11 @@
           <t>Evasión +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S77" t="inlineStr"/>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>eva:3</t>
+        </is>
+      </c>
       <c r="T77" t="inlineStr"/>
       <c r="U77" t="inlineStr"/>
     </row>
@@ -6110,7 +6198,11 @@
           <t>Movimiento +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S78" t="inlineStr"/>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>mov:3</t>
+        </is>
+      </c>
       <c r="T78" t="inlineStr"/>
       <c r="U78" t="inlineStr"/>
     </row>
@@ -6183,7 +6275,11 @@
           <t>Probabilidad de Golpe +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S79" t="inlineStr"/>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>pdg:3</t>
+        </is>
+      </c>
       <c r="T79" t="inlineStr"/>
       <c r="U79" t="inlineStr"/>
     </row>
@@ -6256,7 +6352,11 @@
           <t>Rango +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S80" t="inlineStr"/>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>rng:3</t>
+        </is>
+      </c>
       <c r="T80" t="inlineStr"/>
       <c r="U80" t="inlineStr"/>
     </row>
@@ -6329,7 +6429,11 @@
           <t>Parry +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S81" t="inlineStr"/>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>parry:3</t>
+        </is>
+      </c>
       <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr"/>
     </row>
@@ -6402,7 +6506,11 @@
           <t>Bonos máximos +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S82" t="inlineStr"/>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>bonos:3</t>
+        </is>
+      </c>
       <c r="T82" t="inlineStr"/>
       <c r="U82" t="inlineStr"/>
     </row>
@@ -6475,7 +6583,11 @@
           <t>HP máximo +30. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S83" t="inlineStr"/>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>hpmax:30</t>
+        </is>
+      </c>
       <c r="T83" t="inlineStr"/>
       <c r="U83" t="inlineStr"/>
     </row>
@@ -6548,7 +6660,11 @@
           <t>Resistencia a CC +3. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S84" t="inlineStr"/>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>rescc:3</t>
+        </is>
+      </c>
       <c r="T84" t="inlineStr"/>
       <c r="U84" t="inlineStr"/>
     </row>
@@ -7177,7 +7293,11 @@
           <t>Resistencia mágica +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S93" t="inlineStr"/>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>resmg:2</t>
+        </is>
+      </c>
       <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr"/>
     </row>
@@ -7250,7 +7370,11 @@
           <t>Rango de Casteo +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S94" t="inlineStr"/>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>rangocasteo:2</t>
+        </is>
+      </c>
       <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr"/>
     </row>
@@ -7323,7 +7447,11 @@
           <t>Probabilidad de golpe mágico +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S95" t="inlineStr"/>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>pdgmg:2</t>
+        </is>
+      </c>
       <c r="T95" t="inlineStr"/>
       <c r="U95" t="inlineStr"/>
     </row>
@@ -7396,7 +7524,11 @@
           <t>Daño +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S96" t="inlineStr"/>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>dmg:2</t>
+        </is>
+      </c>
       <c r="T96" t="inlineStr"/>
       <c r="U96" t="inlineStr"/>
     </row>
@@ -7469,7 +7601,11 @@
           <t>Bloqueo +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S97" t="inlineStr"/>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>bloqueo:2</t>
+        </is>
+      </c>
       <c r="T97" t="inlineStr"/>
       <c r="U97" t="inlineStr"/>
     </row>
@@ -7542,7 +7678,11 @@
           <t>Crítico +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S98" t="inlineStr"/>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>crit:2</t>
+        </is>
+      </c>
       <c r="T98" t="inlineStr"/>
       <c r="U98" t="inlineStr"/>
     </row>
@@ -7615,7 +7755,11 @@
           <t>Evasión +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S99" t="inlineStr"/>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>eva:2</t>
+        </is>
+      </c>
       <c r="T99" t="inlineStr"/>
       <c r="U99" t="inlineStr"/>
     </row>
@@ -7688,7 +7832,11 @@
           <t>Movimiento +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S100" t="inlineStr"/>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>mov:2</t>
+        </is>
+      </c>
       <c r="T100" t="inlineStr"/>
       <c r="U100" t="inlineStr"/>
     </row>
@@ -7761,7 +7909,11 @@
           <t>Probabilidad de Golpe +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S101" t="inlineStr"/>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>pdg:2</t>
+        </is>
+      </c>
       <c r="T101" t="inlineStr"/>
       <c r="U101" t="inlineStr"/>
     </row>
@@ -7834,7 +7986,11 @@
           <t>Rango +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S102" t="inlineStr"/>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>rng:2</t>
+        </is>
+      </c>
       <c r="T102" t="inlineStr"/>
       <c r="U102" t="inlineStr"/>
     </row>
@@ -7907,7 +8063,11 @@
           <t>Parry +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S103" t="inlineStr"/>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>parry:2</t>
+        </is>
+      </c>
       <c r="T103" t="inlineStr"/>
       <c r="U103" t="inlineStr"/>
     </row>
@@ -7980,7 +8140,11 @@
           <t>Bonos máximos +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S104" t="inlineStr"/>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>bonos:2</t>
+        </is>
+      </c>
       <c r="T104" t="inlineStr"/>
       <c r="U104" t="inlineStr"/>
     </row>
@@ -8053,7 +8217,11 @@
           <t>HP máximo +20. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S105" t="inlineStr"/>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>hpmax:20</t>
+        </is>
+      </c>
       <c r="T105" t="inlineStr"/>
       <c r="U105" t="inlineStr"/>
     </row>
@@ -8126,7 +8294,11 @@
           <t>Resistencia a CC +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S106" t="inlineStr"/>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>rescc:2</t>
+        </is>
+      </c>
       <c r="T106" t="inlineStr"/>
       <c r="U106" t="inlineStr"/>
     </row>
@@ -8199,7 +8371,11 @@
           <t>Acciones máximas +2. Dura hasta el fin del combate (bórralo a mano al terminar).</t>
         </is>
       </c>
-      <c r="S107" t="inlineStr"/>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>accionesmax:2</t>
+        </is>
+      </c>
       <c r="T107" t="inlineStr"/>
       <c r="U107" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Estados: Pajaritos y Cansado ahora cuentan como CC
Confirmado por el usuario: "Inmunidad a CC" debía cubrir también
Pajaritos y Cansado, no solo Stun/Exhausto. Se les suma esCC:true en
EFECTOS_PRESET (ficha.html) y ESTADOS_PRESET_GM (gm-tools.html).

Esto además termina de automatizar 2 de los anillos "recordatorio" del
commit anterior: Anillo de Inmutabilidad y Anillo de vigor pasan a usar
equipoEstadoPreset: 'Inmunidad a CC' — ahora sí bloquean de verdad lo
que describen (antes no había un preset que cubriera exactamente esa
combinación).
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -24028,7 +24028,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Inmutabilidad (anillo)</t>
+          <t>Inmunidad a CC (anillo)</t>
         </is>
       </c>
       <c r="Q8" t="n">
@@ -24036,10 +24036,14 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Mientras esté equipado, se supone inmune a Stun y a Pajaritos. Recordatorio: no hay un preset que cubra exactamente esta combinación — hay que bloquear esos debuffs a mano si se los intentan aplicar.</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>Inmune a estados de control (Stun, Exhausto, Pajaritos, Cansado): no se le pueden aplicar mientras esté equipado.</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Inmunidad a CC</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
     </row>
@@ -25203,7 +25207,7 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Vigor (anillo)</t>
+          <t>Inmunidad a CC (anillo)</t>
         </is>
       </c>
       <c r="Q25" t="n">
@@ -25211,10 +25215,14 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Mientras esté equipado, se supone inmune a Cansado y Exhausto. Recordatorio: Inmunidad a CC solo cubre Exhausto (Cansado no está tageado como CC) — ese hay que bloqueárselo a mano.</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr"/>
+          <t>Inmune a estados de control (Stun, Exhausto, Pajaritos, Cansado): no se le pueden aplicar mientras esté equipado.</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Inmunidad a CC</t>
+        </is>
+      </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Catálogo: columna "Ocultar en el catálogo" en Defensivos
Nueva columna (booleana, como Legacy) para ítems generados en automático
que todavía no se auditaron/balancearon. Los marcados "sí" no se
escriben a ficha.html, vendor-generator.html ni gm-tools.html —no se
pueden comprar, ni aparecen en tiendas generadas, ni se pueden equipar
en un creep— pero siguen enteros en datos/catalogo.json y en el Excel
para poder editarlos y, cuando estén listos, destildarlos.

Por ahora solo en la pestaña Defensivos, que es donde hacía falta.
importar.py/importar_json.py avisan cuántos y cuáles ítems quedaron
ocultos en cada corrida.
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Consumibles'!$A$1:$U$130</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$W$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Escudos'!$A$1:$U$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defensivos'!$A$1:$AH$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defensivos'!$A$1:$AI$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Accesorios'!$A$1:$U$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Otros'!$A$1:$Q$2</definedName>
   </definedNames>
@@ -16814,7 +16814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH95"/>
+  <dimension ref="A1:AI95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16849,8 +16849,9 @@
     <col width="13" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
     <col width="13" customWidth="1" min="32" max="32"/>
-    <col width="30" customWidth="1" min="33" max="33"/>
-    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="30" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16896,130 +16897,135 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
+          <t>Ocultar en el catálogo</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
           <t>Defensa</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Res.Crít Tipo 2</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Res.Crít Tipo 4</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Res.Crít Tipo 6</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Res.Crít Tipo 8</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Res.Crít Tipo 10</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Movimiento</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Bonos</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>Evasión</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>Iniciativa</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>PdG</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>Parry</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>Fuerza</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>Constitución</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>Inteligencia</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>Destreza</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>Agilidad</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>Res. mental</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>Res. CC</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>Rango casteo</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>Acciones máx.</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>Estado al equipar</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>HP por turno equipado</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>Detalle del estado equipado</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>Otros modificadores</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Tiene imagen</t>
         </is>
@@ -17060,10 +17066,10 @@
           <t>Reduce críticos tipo 6 y 8</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="n">
         <v>8</v>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
@@ -17084,12 +17090,13 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17126,16 +17133,16 @@
           <t>Reduce críticos Tipo 2 y 4.</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="n">
         <v>3</v>
       </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
       <c r="K3" t="n">
         <v>1</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
@@ -17154,12 +17161,13 @@
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="n">
+        <v>0</v>
+      </c>
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17196,10 +17204,10 @@
           <t>Reduce críticos tipo 4 y 6</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
         <v>7</v>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
@@ -17220,12 +17228,13 @@
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
       <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -17258,20 +17267,20 @@
         <v>90</v>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="n">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
         <v>4</v>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
       <c r="N5" t="inlineStr"/>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
@@ -17286,12 +17295,13 @@
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
       <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -17324,17 +17334,17 @@
         <v>93</v>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="n">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
         <v>6</v>
       </c>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
@@ -17352,12 +17362,13 @@
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -17390,10 +17401,10 @@
         <v>110</v>
       </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="n">
         <v>5</v>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
@@ -17414,12 +17425,13 @@
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
       <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17456,10 +17468,10 @@
           <t>Ranuras para consumibles +1</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
@@ -17480,16 +17492,17 @@
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr">
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr">
         <is>
           <t>capcinturon:1</t>
         </is>
       </c>
-      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17548,16 +17561,17 @@
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr">
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr">
         <is>
           <t>capcinturon:3</t>
         </is>
       </c>
-      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17594,19 +17608,19 @@
           <t>Reduce críticos Tipo 2, 4 y 6.</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
         <v>5</v>
       </c>
-      <c r="J10" t="n">
-        <v>1</v>
-      </c>
       <c r="K10" t="n">
         <v>1</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
@@ -17624,12 +17638,13 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -17666,10 +17681,10 @@
           <t>Reduce críticos tipo 4</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="n">
         <v>3</v>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
@@ -17690,12 +17705,13 @@
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17732,18 +17748,18 @@
           <t>Reduce críticos Tipo 6 y 8.</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="n">
         <v>6</v>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="n">
-        <v>1</v>
-      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
         <v>1</v>
       </c>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
@@ -17760,12 +17776,13 @@
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="n">
+        <v>0</v>
+      </c>
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -17802,19 +17819,19 @@
           <t>Reduce críticos Tipo 2, 4 y 6.</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="n">
         <v>5</v>
       </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
       <c r="K13" t="n">
         <v>1</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
@@ -17832,12 +17849,13 @@
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="n">
+        <v>0</v>
+      </c>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17874,17 +17892,17 @@
           <t>Reduce críticos Tipo 4 y 6.</t>
         </is>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="n">
         <v>4</v>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="n">
-        <v>1</v>
-      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>1</v>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
@@ -17902,12 +17920,13 @@
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="n">
+        <v>0</v>
+      </c>
       <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -17944,16 +17963,16 @@
           <t>Reduce críticos Tipo 2 y 4.</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="n">
         <v>3</v>
       </c>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
       <c r="K15" t="n">
         <v>1</v>
       </c>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
@@ -17972,12 +17991,13 @@
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="n">
+        <v>0</v>
+      </c>
       <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -18014,13 +18034,13 @@
           <t>Buen agarre para trepar y colgar de un acantilado.</t>
         </is>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="n">
         <v>2</v>
       </c>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -18028,10 +18048,10 @@
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
-      <c r="S16" t="n">
-        <v>1</v>
-      </c>
-      <c r="T16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="n">
+        <v>1</v>
+      </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
@@ -18042,12 +18062,13 @@
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="n">
+        <v>0</v>
+      </c>
       <c r="AG16" t="inlineStr"/>
       <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -18084,17 +18105,17 @@
           <t>Reduce críticos Tipo 4 y 6.</t>
         </is>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="n">
         <v>5</v>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="n">
-        <v>1</v>
-      </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>1</v>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
@@ -18112,12 +18133,13 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="n">
+        <v>0</v>
+      </c>
       <c r="AG17" t="inlineStr"/>
       <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -18154,16 +18176,16 @@
           <t>Reduce críticos Tipo 2 y 4.</t>
         </is>
       </c>
-      <c r="I18" t="n">
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="n">
         <v>4</v>
       </c>
-      <c r="J18" t="n">
-        <v>1</v>
-      </c>
       <c r="K18" t="n">
         <v>1</v>
       </c>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
@@ -18182,12 +18204,13 @@
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="n">
+        <v>0</v>
+      </c>
       <c r="AG18" t="inlineStr"/>
       <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -18224,20 +18247,20 @@
           <t>Reduce críticos tipo 6</t>
         </is>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="n">
         <v>4</v>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="n">
-        <v>1</v>
-      </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="n">
+        <v>1</v>
+      </c>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
@@ -18252,12 +18275,13 @@
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="n">
+        <v>0</v>
+      </c>
       <c r="AG19" t="inlineStr"/>
       <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -18290,18 +18314,18 @@
         <v>111</v>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
         <v>7</v>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="n">
-        <v>1</v>
-      </c>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
         <v>1</v>
       </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
@@ -18318,12 +18342,13 @@
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="n">
+        <v>0</v>
+      </c>
       <c r="AG20" t="inlineStr"/>
       <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -18360,24 +18385,24 @@
           <t>Reduce críticos Tipo 4, 6 y 8. -1 Movimiento.</t>
         </is>
       </c>
-      <c r="I21" t="n">
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
         <v>6</v>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="n">
-        <v>1</v>
-      </c>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="n">
+      <c r="N21" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="n">
         <v>-1</v>
       </c>
-      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
@@ -18392,12 +18417,13 @@
       <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="inlineStr"/>
       <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="n">
+        <v>0</v>
+      </c>
       <c r="AG21" t="inlineStr"/>
       <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -18430,14 +18456,14 @@
         <v>92</v>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
         <v>4</v>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
@@ -18453,17 +18479,18 @@
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="n">
+        <v>1</v>
+      </c>
       <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="n">
+        <v>0</v>
+      </c>
       <c r="AG22" t="inlineStr"/>
       <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -18500,20 +18527,20 @@
           <t>Reduce críticos Tipo 2, 6 y 8.</t>
         </is>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="n">
         <v>6</v>
       </c>
-      <c r="J23" t="n">
-        <v>1</v>
-      </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="n">
-        <v>1</v>
-      </c>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
         <v>1</v>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>1</v>
+      </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
@@ -18530,12 +18557,13 @@
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="n">
+        <v>0</v>
+      </c>
       <c r="AG23" t="inlineStr"/>
       <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -18568,18 +18596,18 @@
         <v>98</v>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="n">
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="n">
         <v>6</v>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="n">
-        <v>1</v>
-      </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
@@ -18596,12 +18624,13 @@
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="n">
+        <v>0</v>
+      </c>
       <c r="AG24" t="inlineStr"/>
       <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -18638,18 +18667,18 @@
           <t>Reduce críticos Tipo 6 y 8.</t>
         </is>
       </c>
-      <c r="I25" t="n">
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="n">
         <v>5</v>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="n">
-        <v>1</v>
-      </c>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
         <v>1</v>
       </c>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>1</v>
+      </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
@@ -18666,12 +18695,13 @@
       <c r="AB25" t="inlineStr"/>
       <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
       <c r="AG25" t="inlineStr"/>
       <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -18704,10 +18734,10 @@
         <v>50</v>
       </c>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="n">
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="n">
         <v>3</v>
       </c>
-      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
@@ -18728,12 +18758,13 @@
       <c r="AB26" t="inlineStr"/>
       <c r="AC26" t="inlineStr"/>
       <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
       <c r="AG26" t="inlineStr"/>
       <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -18770,20 +18801,20 @@
           <t>Reduce críticos Tipo 2 y 4</t>
         </is>
       </c>
-      <c r="I27" t="n">
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="n">
         <v>4</v>
       </c>
-      <c r="J27" t="n">
-        <v>1</v>
-      </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="n">
-        <v>1</v>
-      </c>
-      <c r="N27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
@@ -18800,12 +18831,13 @@
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr"/>
-      <c r="AE27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="n">
+        <v>0</v>
+      </c>
       <c r="AG27" t="inlineStr"/>
       <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -18842,10 +18874,10 @@
           <t>Reduce críticos tipo 2</t>
         </is>
       </c>
-      <c r="I28" t="n">
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="n">
         <v>3</v>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
@@ -18866,12 +18898,13 @@
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
       <c r="AD28" t="inlineStr"/>
-      <c r="AE28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="n">
+        <v>0</v>
+      </c>
       <c r="AG28" t="inlineStr"/>
       <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -18904,16 +18937,16 @@
         <v>37</v>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="n">
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="n">
         <v>3</v>
       </c>
-      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
-      <c r="M29" t="n">
-        <v>1</v>
-      </c>
-      <c r="N29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="n">
+        <v>1</v>
+      </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
@@ -18930,12 +18963,13 @@
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="inlineStr"/>
       <c r="AD29" t="inlineStr"/>
-      <c r="AE29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="n">
+        <v>0</v>
+      </c>
       <c r="AG29" t="inlineStr"/>
       <c r="AH29" t="inlineStr"/>
+      <c r="AI29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -18968,16 +19002,16 @@
         <v>41</v>
       </c>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="n">
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="n">
         <v>4</v>
       </c>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
-      <c r="M30" t="n">
-        <v>1</v>
-      </c>
-      <c r="N30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="n">
+        <v>1</v>
+      </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
@@ -18994,12 +19028,13 @@
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr"/>
       <c r="AD30" t="inlineStr"/>
-      <c r="AE30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
       <c r="AG30" t="inlineStr"/>
       <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -19032,18 +19067,18 @@
         <v>38</v>
       </c>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="n">
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="n">
         <v>2</v>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
-      <c r="O31" t="n">
-        <v>1</v>
-      </c>
-      <c r="P31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>1</v>
+      </c>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
@@ -19058,12 +19093,13 @@
       <c r="AB31" t="inlineStr"/>
       <c r="AC31" t="inlineStr"/>
       <c r="AD31" t="inlineStr"/>
-      <c r="AE31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
       <c r="AG31" t="inlineStr"/>
       <c r="AH31" t="inlineStr"/>
+      <c r="AI31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -19100,15 +19136,15 @@
           <t>Reduce críticos Tipo 6.</t>
         </is>
       </c>
-      <c r="I32" t="n">
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="n">
         <v>3</v>
       </c>
-      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="n">
-        <v>1</v>
-      </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>1</v>
+      </c>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
@@ -19126,12 +19162,13 @@
       <c r="AB32" t="inlineStr"/>
       <c r="AC32" t="inlineStr"/>
       <c r="AD32" t="inlineStr"/>
-      <c r="AE32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="n">
+        <v>0</v>
+      </c>
       <c r="AG32" t="inlineStr"/>
       <c r="AH32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -19164,10 +19201,10 @@
         <v>70</v>
       </c>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
@@ -19188,12 +19225,13 @@
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr"/>
       <c r="AD33" t="inlineStr"/>
-      <c r="AE33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
       <c r="AG33" t="inlineStr"/>
       <c r="AH33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -19226,13 +19264,13 @@
         <v>32</v>
       </c>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="n">
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="n">
         <v>2</v>
       </c>
-      <c r="J34" t="n">
-        <v>1</v>
-      </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="n">
+        <v>1</v>
+      </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
@@ -19252,12 +19290,13 @@
       <c r="AB34" t="inlineStr"/>
       <c r="AC34" t="inlineStr"/>
       <c r="AD34" t="inlineStr"/>
-      <c r="AE34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr"/>
+      <c r="AF34" t="n">
+        <v>0</v>
+      </c>
       <c r="AG34" t="inlineStr"/>
       <c r="AH34" t="inlineStr"/>
+      <c r="AI34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -19290,10 +19329,10 @@
         <v>40</v>
       </c>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="n">
-        <v>1</v>
-      </c>
-      <c r="J35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -19314,12 +19353,13 @@
       <c r="AB35" t="inlineStr"/>
       <c r="AC35" t="inlineStr"/>
       <c r="AD35" t="inlineStr"/>
-      <c r="AE35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF35" t="inlineStr"/>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="n">
+        <v>0</v>
+      </c>
       <c r="AG35" t="inlineStr"/>
       <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -19352,15 +19392,15 @@
         <v>70</v>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="n">
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="n">
         <v>4</v>
       </c>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="n">
-        <v>1</v>
-      </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>1</v>
+      </c>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
@@ -19378,12 +19418,13 @@
       <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="inlineStr"/>
       <c r="AD36" t="inlineStr"/>
-      <c r="AE36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
+      <c r="AF36" t="n">
+        <v>0</v>
+      </c>
       <c r="AG36" t="inlineStr"/>
       <c r="AH36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -19416,16 +19457,16 @@
         <v>42</v>
       </c>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="n">
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="n">
         <v>3</v>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
-      <c r="M37" t="n">
-        <v>1</v>
-      </c>
-      <c r="N37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="n">
+        <v>1</v>
+      </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
@@ -19442,12 +19483,13 @@
       <c r="AB37" t="inlineStr"/>
       <c r="AC37" t="inlineStr"/>
       <c r="AD37" t="inlineStr"/>
-      <c r="AE37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF37" t="inlineStr"/>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="n">
+        <v>0</v>
+      </c>
       <c r="AG37" t="inlineStr"/>
       <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -19480,16 +19522,16 @@
         <v>37</v>
       </c>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="n">
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="n">
         <v>3</v>
       </c>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="n">
-        <v>1</v>
-      </c>
-      <c r="N38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="n">
+        <v>1</v>
+      </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
@@ -19506,12 +19548,13 @@
       <c r="AB38" t="inlineStr"/>
       <c r="AC38" t="inlineStr"/>
       <c r="AD38" t="inlineStr"/>
-      <c r="AE38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF38" t="inlineStr"/>
+      <c r="AE38" t="inlineStr"/>
+      <c r="AF38" t="n">
+        <v>0</v>
+      </c>
       <c r="AG38" t="inlineStr"/>
       <c r="AH38" t="inlineStr"/>
+      <c r="AI38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -19544,13 +19587,13 @@
         <v>37</v>
       </c>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="n">
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="n">
         <v>2</v>
       </c>
-      <c r="J39" t="n">
-        <v>1</v>
-      </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" t="n">
+        <v>1</v>
+      </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
@@ -19570,12 +19613,13 @@
       <c r="AB39" t="inlineStr"/>
       <c r="AC39" t="inlineStr"/>
       <c r="AD39" t="inlineStr"/>
-      <c r="AE39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF39" t="inlineStr"/>
+      <c r="AE39" t="inlineStr"/>
+      <c r="AF39" t="n">
+        <v>0</v>
+      </c>
       <c r="AG39" t="inlineStr"/>
       <c r="AH39" t="inlineStr"/>
+      <c r="AI39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -19612,16 +19656,16 @@
           <t>Reduce críticos Tipo 8.</t>
         </is>
       </c>
-      <c r="I40" t="n">
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="n">
         <v>3</v>
       </c>
-      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
-      <c r="M40" t="n">
-        <v>1</v>
-      </c>
-      <c r="N40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="n">
+        <v>1</v>
+      </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
@@ -19638,12 +19682,13 @@
       <c r="AB40" t="inlineStr"/>
       <c r="AC40" t="inlineStr"/>
       <c r="AD40" t="inlineStr"/>
-      <c r="AE40" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF40" t="inlineStr"/>
+      <c r="AE40" t="inlineStr"/>
+      <c r="AF40" t="n">
+        <v>0</v>
+      </c>
       <c r="AG40" t="inlineStr"/>
       <c r="AH40" t="inlineStr"/>
+      <c r="AI40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -19676,16 +19721,16 @@
         <v>56</v>
       </c>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="n">
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="n">
         <v>5</v>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
-      <c r="M41" t="n">
-        <v>1</v>
-      </c>
-      <c r="N41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="n">
+        <v>1</v>
+      </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
@@ -19702,12 +19747,13 @@
       <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="inlineStr"/>
       <c r="AD41" t="inlineStr"/>
-      <c r="AE41" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF41" t="inlineStr"/>
+      <c r="AE41" t="inlineStr"/>
+      <c r="AF41" t="n">
+        <v>0</v>
+      </c>
       <c r="AG41" t="inlineStr"/>
       <c r="AH41" t="inlineStr"/>
+      <c r="AI41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -19766,16 +19812,17 @@
       <c r="AB42" t="inlineStr"/>
       <c r="AC42" t="inlineStr"/>
       <c r="AD42" t="inlineStr"/>
-      <c r="AE42" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF42" t="inlineStr"/>
-      <c r="AG42" t="inlineStr">
+      <c r="AE42" t="inlineStr"/>
+      <c r="AF42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr">
         <is>
           <t>capcinturon:1</t>
         </is>
       </c>
-      <c r="AH42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -19812,18 +19859,18 @@
           <t>Reduce críticos tipo 4, 6 y 8</t>
         </is>
       </c>
-      <c r="I43" t="n">
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="n">
         <v>8</v>
       </c>
-      <c r="J43" t="n">
-        <v>1</v>
-      </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="n">
+        <v>1</v>
+      </c>
       <c r="L43" t="inlineStr"/>
-      <c r="M43" t="n">
-        <v>1</v>
-      </c>
-      <c r="N43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="n">
+        <v>1</v>
+      </c>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
@@ -19840,12 +19887,13 @@
       <c r="AB43" t="inlineStr"/>
       <c r="AC43" t="inlineStr"/>
       <c r="AD43" t="inlineStr"/>
-      <c r="AE43" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
+      <c r="AF43" t="n">
+        <v>0</v>
+      </c>
       <c r="AG43" t="inlineStr"/>
       <c r="AH43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -19882,10 +19930,10 @@
           <t>Reduce críticos Tipo 2, 4 y 6.</t>
         </is>
       </c>
-      <c r="I44" t="n">
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="n">
         <v>5</v>
       </c>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
@@ -19906,12 +19954,13 @@
       <c r="AB44" t="inlineStr"/>
       <c r="AC44" t="inlineStr"/>
       <c r="AD44" t="inlineStr"/>
-      <c r="AE44" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF44" t="inlineStr"/>
+      <c r="AE44" t="inlineStr"/>
+      <c r="AF44" t="n">
+        <v>0</v>
+      </c>
       <c r="AG44" t="inlineStr"/>
       <c r="AH44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -19944,16 +19993,16 @@
         <v>42</v>
       </c>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="n">
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="n">
         <v>3</v>
       </c>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
-      <c r="M45" t="n">
-        <v>1</v>
-      </c>
-      <c r="N45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="n">
+        <v>1</v>
+      </c>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
@@ -19970,12 +20019,13 @@
       <c r="AB45" t="inlineStr"/>
       <c r="AC45" t="inlineStr"/>
       <c r="AD45" t="inlineStr"/>
-      <c r="AE45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF45" t="inlineStr"/>
+      <c r="AE45" t="inlineStr"/>
+      <c r="AF45" t="n">
+        <v>0</v>
+      </c>
       <c r="AG45" t="inlineStr"/>
       <c r="AH45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -20008,16 +20058,16 @@
         <v>46</v>
       </c>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="n">
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="n">
         <v>4</v>
       </c>
-      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
-      <c r="M46" t="n">
-        <v>1</v>
-      </c>
-      <c r="N46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="n">
+        <v>1</v>
+      </c>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
@@ -20034,12 +20084,13 @@
       <c r="AB46" t="inlineStr"/>
       <c r="AC46" t="inlineStr"/>
       <c r="AD46" t="inlineStr"/>
-      <c r="AE46" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF46" t="inlineStr"/>
+      <c r="AE46" t="inlineStr"/>
+      <c r="AF46" t="n">
+        <v>0</v>
+      </c>
       <c r="AG46" t="inlineStr"/>
       <c r="AH46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -20076,17 +20127,17 @@
           <t>Reduce críticos Tipo 2.</t>
         </is>
       </c>
-      <c r="I47" t="n">
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="n">
         <v>2</v>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="n">
-        <v>1</v>
-      </c>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" t="n">
         <v>1</v>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="n">
+        <v>1</v>
+      </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
@@ -20104,12 +20155,13 @@
       <c r="AB47" t="inlineStr"/>
       <c r="AC47" t="inlineStr"/>
       <c r="AD47" t="inlineStr"/>
-      <c r="AE47" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF47" t="inlineStr"/>
+      <c r="AE47" t="inlineStr"/>
+      <c r="AF47" t="n">
+        <v>0</v>
+      </c>
       <c r="AG47" t="inlineStr"/>
       <c r="AH47" t="inlineStr"/>
+      <c r="AI47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -20146,20 +20198,20 @@
           <t>Reduce críticos Tipo 2 y 4. Reduce en 1 el daño de fuego.</t>
         </is>
       </c>
-      <c r="I48" t="n">
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="n">
         <v>4</v>
       </c>
-      <c r="J48" t="n">
-        <v>1</v>
-      </c>
       <c r="K48" t="n">
         <v>1</v>
       </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="n">
-        <v>1</v>
-      </c>
-      <c r="N48" t="inlineStr"/>
+      <c r="L48" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="n">
+        <v>1</v>
+      </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
@@ -20176,12 +20228,13 @@
       <c r="AB48" t="inlineStr"/>
       <c r="AC48" t="inlineStr"/>
       <c r="AD48" t="inlineStr"/>
-      <c r="AE48" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF48" t="inlineStr"/>
+      <c r="AE48" t="inlineStr"/>
+      <c r="AF48" t="n">
+        <v>0</v>
+      </c>
       <c r="AG48" t="inlineStr"/>
       <c r="AH48" t="inlineStr"/>
+      <c r="AI48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -20214,14 +20267,14 @@
         <v>80</v>
       </c>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="n">
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="n">
         <v>2</v>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="n">
-        <v>1</v>
-      </c>
-      <c r="L49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="n">
+        <v>1</v>
+      </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
@@ -20240,12 +20293,13 @@
       <c r="AB49" t="inlineStr"/>
       <c r="AC49" t="inlineStr"/>
       <c r="AD49" t="inlineStr"/>
-      <c r="AE49" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr"/>
+      <c r="AF49" t="n">
+        <v>0</v>
+      </c>
       <c r="AG49" t="inlineStr"/>
       <c r="AH49" t="inlineStr"/>
+      <c r="AI49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -20278,18 +20332,18 @@
         <v>34</v>
       </c>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="n">
-        <v>1</v>
-      </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
-      <c r="O50" t="n">
-        <v>1</v>
-      </c>
-      <c r="P50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="n">
+        <v>1</v>
+      </c>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr"/>
@@ -20304,12 +20358,13 @@
       <c r="AB50" t="inlineStr"/>
       <c r="AC50" t="inlineStr"/>
       <c r="AD50" t="inlineStr"/>
-      <c r="AE50" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="n">
+        <v>0</v>
+      </c>
       <c r="AG50" t="inlineStr"/>
       <c r="AH50" t="inlineStr"/>
+      <c r="AI50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -20346,16 +20401,16 @@
           <t>Reduce en 1 el daño de fuego.</t>
         </is>
       </c>
-      <c r="I51" t="n">
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="n">
         <v>3</v>
       </c>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
-      <c r="M51" t="n">
-        <v>1</v>
-      </c>
-      <c r="N51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="n">
+        <v>1</v>
+      </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
@@ -20372,12 +20427,13 @@
       <c r="AB51" t="inlineStr"/>
       <c r="AC51" t="inlineStr"/>
       <c r="AD51" t="inlineStr"/>
-      <c r="AE51" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr"/>
+      <c r="AF51" t="n">
+        <v>0</v>
+      </c>
       <c r="AG51" t="inlineStr"/>
       <c r="AH51" t="inlineStr"/>
+      <c r="AI51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -20414,19 +20470,19 @@
           <t>Tejido con patrones florales. Muy abrigaditos.</t>
         </is>
       </c>
-      <c r="I52" t="n">
-        <v>1</v>
-      </c>
-      <c r="J52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="n">
+        <v>1</v>
+      </c>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="n">
+        <v>1</v>
+      </c>
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
@@ -20440,12 +20496,13 @@
       <c r="AB52" t="inlineStr"/>
       <c r="AC52" t="inlineStr"/>
       <c r="AD52" t="inlineStr"/>
-      <c r="AE52" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr"/>
+      <c r="AF52" t="n">
+        <v>0</v>
+      </c>
       <c r="AG52" t="inlineStr"/>
       <c r="AH52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -20478,18 +20535,18 @@
         <v>34</v>
       </c>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="n">
-        <v>1</v>
-      </c>
-      <c r="J53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="n">
+        <v>1</v>
+      </c>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
-      <c r="O53" t="n">
-        <v>1</v>
-      </c>
-      <c r="P53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="n">
+        <v>1</v>
+      </c>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr"/>
       <c r="S53" t="inlineStr"/>
@@ -20504,12 +20561,13 @@
       <c r="AB53" t="inlineStr"/>
       <c r="AC53" t="inlineStr"/>
       <c r="AD53" t="inlineStr"/>
-      <c r="AE53" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF53" t="inlineStr"/>
+      <c r="AE53" t="inlineStr"/>
+      <c r="AF53" t="n">
+        <v>0</v>
+      </c>
       <c r="AG53" t="inlineStr"/>
       <c r="AH53" t="inlineStr"/>
+      <c r="AI53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -20546,13 +20604,13 @@
           <t>Reduce críticos Tipo 2.</t>
         </is>
       </c>
-      <c r="I54" t="n">
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="n">
         <v>3</v>
       </c>
-      <c r="J54" t="n">
-        <v>1</v>
-      </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="n">
+        <v>1</v>
+      </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
@@ -20572,12 +20630,13 @@
       <c r="AB54" t="inlineStr"/>
       <c r="AC54" t="inlineStr"/>
       <c r="AD54" t="inlineStr"/>
-      <c r="AE54" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF54" t="inlineStr"/>
+      <c r="AE54" t="inlineStr"/>
+      <c r="AF54" t="n">
+        <v>0</v>
+      </c>
       <c r="AG54" t="inlineStr"/>
       <c r="AH54" t="inlineStr"/>
+      <c r="AI54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -20610,13 +20669,13 @@
         <v>90</v>
       </c>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="n">
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="n">
         <v>4</v>
       </c>
-      <c r="J55" t="n">
-        <v>1</v>
-      </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="K55" t="n">
+        <v>1</v>
+      </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
@@ -20636,12 +20695,13 @@
       <c r="AB55" t="inlineStr"/>
       <c r="AC55" t="inlineStr"/>
       <c r="AD55" t="inlineStr"/>
-      <c r="AE55" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF55" t="inlineStr"/>
+      <c r="AE55" t="inlineStr"/>
+      <c r="AF55" t="n">
+        <v>0</v>
+      </c>
       <c r="AG55" t="inlineStr"/>
       <c r="AH55" t="inlineStr"/>
+      <c r="AI55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -20678,16 +20738,16 @@
           <t>Reduce críticos tipo 4 y 6</t>
         </is>
       </c>
-      <c r="I56" t="n">
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="n">
         <v>5</v>
       </c>
-      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
-      <c r="M56" t="n">
-        <v>1</v>
-      </c>
-      <c r="N56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="n">
+        <v>1</v>
+      </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="inlineStr"/>
@@ -20704,12 +20764,13 @@
       <c r="AB56" t="inlineStr"/>
       <c r="AC56" t="inlineStr"/>
       <c r="AD56" t="inlineStr"/>
-      <c r="AE56" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF56" t="inlineStr"/>
+      <c r="AE56" t="inlineStr"/>
+      <c r="AF56" t="n">
+        <v>0</v>
+      </c>
       <c r="AG56" t="inlineStr"/>
       <c r="AH56" t="inlineStr"/>
+      <c r="AI56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -20746,16 +20807,16 @@
           <t>Reduce críticos tipo 6 y 8</t>
         </is>
       </c>
-      <c r="I57" t="n">
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="n">
         <v>6</v>
       </c>
-      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
-      <c r="M57" t="n">
-        <v>1</v>
-      </c>
-      <c r="N57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="n">
+        <v>1</v>
+      </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="inlineStr"/>
@@ -20772,12 +20833,13 @@
       <c r="AB57" t="inlineStr"/>
       <c r="AC57" t="inlineStr"/>
       <c r="AD57" t="inlineStr"/>
-      <c r="AE57" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr"/>
+      <c r="AF57" t="n">
+        <v>0</v>
+      </c>
       <c r="AG57" t="inlineStr"/>
       <c r="AH57" t="inlineStr"/>
+      <c r="AI57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -20814,19 +20876,19 @@
           <t>+1 a los Bonos máximos.</t>
         </is>
       </c>
-      <c r="I58" t="n">
-        <v>1</v>
-      </c>
-      <c r="J58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="n">
+        <v>1</v>
+      </c>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr"/>
@@ -20840,12 +20902,13 @@
       <c r="AB58" t="inlineStr"/>
       <c r="AC58" t="inlineStr"/>
       <c r="AD58" t="inlineStr"/>
-      <c r="AE58" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF58" t="inlineStr"/>
+      <c r="AE58" t="inlineStr"/>
+      <c r="AF58" t="n">
+        <v>0</v>
+      </c>
       <c r="AG58" t="inlineStr"/>
       <c r="AH58" t="inlineStr"/>
+      <c r="AI58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -20882,10 +20945,10 @@
           <t>resistencia mental +5, resistencia mágica +5, resistencia a cc +5</t>
         </is>
       </c>
-      <c r="I59" t="n">
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="n">
         <v>3</v>
       </c>
-      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
@@ -20906,12 +20969,13 @@
       <c r="AB59" t="inlineStr"/>
       <c r="AC59" t="inlineStr"/>
       <c r="AD59" t="inlineStr"/>
-      <c r="AE59" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF59" t="inlineStr"/>
+      <c r="AE59" t="inlineStr"/>
+      <c r="AF59" t="n">
+        <v>0</v>
+      </c>
       <c r="AG59" t="inlineStr"/>
       <c r="AH59" t="inlineStr"/>
+      <c r="AI59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -20970,16 +21034,17 @@
       <c r="AB60" t="inlineStr"/>
       <c r="AC60" t="inlineStr"/>
       <c r="AD60" t="inlineStr"/>
-      <c r="AE60" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF60" t="inlineStr"/>
-      <c r="AG60" t="inlineStr">
+      <c r="AE60" t="inlineStr"/>
+      <c r="AF60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG60" t="inlineStr"/>
+      <c r="AH60" t="inlineStr">
         <is>
           <t>capcinturon:10</t>
         </is>
       </c>
-      <c r="AH60" t="inlineStr"/>
+      <c r="AI60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -21016,16 +21081,16 @@
           <t>Reduce críticos de cualquier tipo.</t>
         </is>
       </c>
-      <c r="I61" t="n">
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="n">
         <v>10</v>
       </c>
-      <c r="J61" t="n">
-        <v>1</v>
-      </c>
       <c r="K61" t="n">
         <v>1</v>
       </c>
-      <c r="L61" t="inlineStr"/>
+      <c r="L61" t="n">
+        <v>1</v>
+      </c>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
@@ -21044,12 +21109,13 @@
       <c r="AB61" t="inlineStr"/>
       <c r="AC61" t="inlineStr"/>
       <c r="AD61" t="inlineStr"/>
-      <c r="AE61" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr"/>
+      <c r="AF61" t="n">
+        <v>0</v>
+      </c>
       <c r="AG61" t="inlineStr"/>
       <c r="AH61" t="inlineStr"/>
+      <c r="AI61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -21086,10 +21152,10 @@
           <t>Reduce críticos Tipo 2, 4 y 6.</t>
         </is>
       </c>
-      <c r="I62" t="n">
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="n">
         <v>7</v>
       </c>
-      <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
@@ -21110,12 +21176,13 @@
       <c r="AB62" t="inlineStr"/>
       <c r="AC62" t="inlineStr"/>
       <c r="AD62" t="inlineStr"/>
-      <c r="AE62" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr"/>
+      <c r="AF62" t="n">
+        <v>0</v>
+      </c>
       <c r="AG62" t="inlineStr"/>
       <c r="AH62" t="inlineStr"/>
+      <c r="AI62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -21152,10 +21219,10 @@
           <t>Otorga regeneración de +3hp x mantenimiento.</t>
         </is>
       </c>
-      <c r="I63" t="n">
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="n">
         <v>4</v>
       </c>
-      <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
@@ -21176,12 +21243,13 @@
       <c r="AB63" t="inlineStr"/>
       <c r="AC63" t="inlineStr"/>
       <c r="AD63" t="inlineStr"/>
-      <c r="AE63" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF63" t="inlineStr"/>
+      <c r="AE63" t="inlineStr"/>
+      <c r="AF63" t="n">
+        <v>0</v>
+      </c>
       <c r="AG63" t="inlineStr"/>
       <c r="AH63" t="inlineStr"/>
+      <c r="AI63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -21218,19 +21286,19 @@
           <t>+1 a los Bonos máximos, +1 Res.M y +1 Res.CC.</t>
         </is>
       </c>
-      <c r="I64" t="n">
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="n">
         <v>2</v>
       </c>
-      <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="n">
+        <v>1</v>
+      </c>
       <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr"/>
@@ -21240,22 +21308,23 @@
       <c r="X64" t="inlineStr"/>
       <c r="Y64" t="inlineStr"/>
       <c r="Z64" t="inlineStr"/>
-      <c r="AA64" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB64" t="inlineStr"/>
+      <c r="AA64" t="inlineStr"/>
+      <c r="AB64" t="n">
+        <v>1</v>
+      </c>
       <c r="AC64" t="inlineStr"/>
       <c r="AD64" t="inlineStr"/>
-      <c r="AE64" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF64" t="inlineStr"/>
-      <c r="AG64" t="inlineStr">
+      <c r="AE64" t="inlineStr"/>
+      <c r="AF64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG64" t="inlineStr"/>
+      <c r="AH64" t="inlineStr">
         <is>
           <t>resmg:1</t>
         </is>
       </c>
-      <c r="AH64" t="inlineStr"/>
+      <c r="AI64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -21292,10 +21361,10 @@
           <t>Ranuras para consumibles +3, inteligencia +1</t>
         </is>
       </c>
-      <c r="I65" t="n">
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="n">
         <v>3</v>
       </c>
-      <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
@@ -21316,12 +21385,13 @@
       <c r="AB65" t="inlineStr"/>
       <c r="AC65" t="inlineStr"/>
       <c r="AD65" t="inlineStr"/>
-      <c r="AE65" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF65" t="inlineStr"/>
+      <c r="AE65" t="inlineStr"/>
+      <c r="AF65" t="n">
+        <v>0</v>
+      </c>
       <c r="AG65" t="inlineStr"/>
       <c r="AH65" t="inlineStr"/>
+      <c r="AI65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -21358,10 +21428,10 @@
           <t>+1 a las Acciones máximas del turno.</t>
         </is>
       </c>
-      <c r="I66" t="n">
-        <v>1</v>
-      </c>
-      <c r="J66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="n">
+        <v>1</v>
+      </c>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
@@ -21380,16 +21450,17 @@
       <c r="Z66" t="inlineStr"/>
       <c r="AA66" t="inlineStr"/>
       <c r="AB66" t="inlineStr"/>
-      <c r="AC66" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD66" t="inlineStr"/>
-      <c r="AE66" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF66" t="inlineStr"/>
+      <c r="AC66" t="inlineStr"/>
+      <c r="AD66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE66" t="inlineStr"/>
+      <c r="AF66" t="n">
+        <v>0</v>
+      </c>
       <c r="AG66" t="inlineStr"/>
       <c r="AH66" t="inlineStr"/>
+      <c r="AI66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -21426,10 +21497,10 @@
           <t>Aura de espinas (de rosas). Regeneración x5hp. Resistencia mágica +5. Cualquier interacción social debe tirar Resistencia Mental para no caer seducidx de manera irrefrenable.</t>
         </is>
       </c>
-      <c r="I67" t="n">
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="n">
         <v>5</v>
       </c>
-      <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr"/>
@@ -21445,19 +21516,20 @@
       <c r="W67" t="inlineStr"/>
       <c r="X67" t="inlineStr"/>
       <c r="Y67" t="inlineStr"/>
-      <c r="Z67" t="n">
+      <c r="Z67" t="inlineStr"/>
+      <c r="AA67" t="n">
         <v>5</v>
       </c>
-      <c r="AA67" t="inlineStr"/>
       <c r="AB67" t="inlineStr"/>
       <c r="AC67" t="inlineStr"/>
       <c r="AD67" t="inlineStr"/>
-      <c r="AE67" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF67" t="inlineStr"/>
+      <c r="AE67" t="inlineStr"/>
+      <c r="AF67" t="n">
+        <v>0</v>
+      </c>
       <c r="AG67" t="inlineStr"/>
       <c r="AH67" t="inlineStr"/>
+      <c r="AI67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -21494,10 +21566,10 @@
           <t>Reduce críticos de cualquier tipo. indestructible</t>
         </is>
       </c>
-      <c r="I68" t="n">
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="n">
         <v>10</v>
       </c>
-      <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
@@ -21518,12 +21590,13 @@
       <c r="AB68" t="inlineStr"/>
       <c r="AC68" t="inlineStr"/>
       <c r="AD68" t="inlineStr"/>
-      <c r="AE68" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF68" t="inlineStr"/>
+      <c r="AE68" t="inlineStr"/>
+      <c r="AF68" t="n">
+        <v>0</v>
+      </c>
       <c r="AG68" t="inlineStr"/>
       <c r="AH68" t="inlineStr"/>
+      <c r="AI68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -21560,10 +21633,10 @@
           <t>Reduce críticos Tipo 2, 4 y 6. Evasión +2. indestructible</t>
         </is>
       </c>
-      <c r="I69" t="n">
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="n">
         <v>10</v>
       </c>
-      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
@@ -21584,12 +21657,13 @@
       <c r="AB69" t="inlineStr"/>
       <c r="AC69" t="inlineStr"/>
       <c r="AD69" t="inlineStr"/>
-      <c r="AE69" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF69" t="inlineStr"/>
+      <c r="AE69" t="inlineStr"/>
+      <c r="AF69" t="n">
+        <v>0</v>
+      </c>
       <c r="AG69" t="inlineStr"/>
       <c r="AH69" t="inlineStr"/>
+      <c r="AI69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -21626,11 +21700,9 @@
           <t>reduce todos los críticos x2</t>
         </is>
       </c>
-      <c r="I70" t="n">
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="n">
         <v>10</v>
-      </c>
-      <c r="J70" t="n">
-        <v>2</v>
       </c>
       <c r="K70" t="n">
         <v>2</v>
@@ -21644,7 +21716,9 @@
       <c r="N70" t="n">
         <v>2</v>
       </c>
-      <c r="O70" t="inlineStr"/>
+      <c r="O70" t="n">
+        <v>2</v>
+      </c>
       <c r="P70" t="inlineStr"/>
       <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr"/>
@@ -21660,12 +21734,13 @@
       <c r="AB70" t="inlineStr"/>
       <c r="AC70" t="inlineStr"/>
       <c r="AD70" t="inlineStr"/>
-      <c r="AE70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF70" t="inlineStr"/>
+      <c r="AE70" t="inlineStr"/>
+      <c r="AF70" t="n">
+        <v>0</v>
+      </c>
       <c r="AG70" t="inlineStr"/>
       <c r="AH70" t="inlineStr"/>
+      <c r="AI70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -21702,10 +21777,10 @@
           <t>destreza +2</t>
         </is>
       </c>
-      <c r="I71" t="n">
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="n">
         <v>3</v>
       </c>
-      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr"/>
@@ -21719,21 +21794,22 @@
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="inlineStr"/>
       <c r="W71" t="inlineStr"/>
-      <c r="X71" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y71" t="inlineStr"/>
+      <c r="X71" t="inlineStr"/>
+      <c r="Y71" t="n">
+        <v>1</v>
+      </c>
       <c r="Z71" t="inlineStr"/>
       <c r="AA71" t="inlineStr"/>
       <c r="AB71" t="inlineStr"/>
       <c r="AC71" t="inlineStr"/>
       <c r="AD71" t="inlineStr"/>
-      <c r="AE71" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF71" t="inlineStr"/>
+      <c r="AE71" t="inlineStr"/>
+      <c r="AF71" t="n">
+        <v>0</v>
+      </c>
       <c r="AG71" t="inlineStr"/>
       <c r="AH71" t="inlineStr"/>
+      <c r="AI71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -21770,10 +21846,10 @@
           <t>inteligencia +2</t>
         </is>
       </c>
-      <c r="I72" t="n">
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="n">
         <v>3</v>
       </c>
-      <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
@@ -21786,22 +21862,23 @@
       <c r="T72" t="inlineStr"/>
       <c r="U72" t="inlineStr"/>
       <c r="V72" t="inlineStr"/>
-      <c r="W72" t="n">
+      <c r="W72" t="inlineStr"/>
+      <c r="X72" t="n">
         <v>2</v>
       </c>
-      <c r="X72" t="inlineStr"/>
       <c r="Y72" t="inlineStr"/>
       <c r="Z72" t="inlineStr"/>
       <c r="AA72" t="inlineStr"/>
       <c r="AB72" t="inlineStr"/>
       <c r="AC72" t="inlineStr"/>
       <c r="AD72" t="inlineStr"/>
-      <c r="AE72" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF72" t="inlineStr"/>
+      <c r="AE72" t="inlineStr"/>
+      <c r="AF72" t="n">
+        <v>0</v>
+      </c>
       <c r="AG72" t="inlineStr"/>
       <c r="AH72" t="inlineStr"/>
+      <c r="AI72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -21838,12 +21915,10 @@
           <t>Resistencia a todos los críticos. +5 a resistencia mágica</t>
         </is>
       </c>
-      <c r="I73" t="n">
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="n">
         <v>5</v>
       </c>
-      <c r="J73" t="n">
-        <v>1</v>
-      </c>
       <c r="K73" t="n">
         <v>1</v>
       </c>
@@ -21856,7 +21931,9 @@
       <c r="N73" t="n">
         <v>1</v>
       </c>
-      <c r="O73" t="inlineStr"/>
+      <c r="O73" t="n">
+        <v>1</v>
+      </c>
       <c r="P73" t="inlineStr"/>
       <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr"/>
@@ -21872,16 +21949,17 @@
       <c r="AB73" t="inlineStr"/>
       <c r="AC73" t="inlineStr"/>
       <c r="AD73" t="inlineStr"/>
-      <c r="AE73" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF73" t="inlineStr"/>
-      <c r="AG73" t="inlineStr">
+      <c r="AE73" t="inlineStr"/>
+      <c r="AF73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG73" t="inlineStr"/>
+      <c r="AH73" t="inlineStr">
         <is>
           <t>resmg:5</t>
         </is>
       </c>
-      <c r="AH73" t="inlineStr"/>
+      <c r="AI73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -21918,10 +21996,10 @@
           <t>Reduce críticos tipo 6 y 8</t>
         </is>
       </c>
-      <c r="I74" t="n">
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="n">
         <v>10</v>
       </c>
-      <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
@@ -21942,12 +22020,13 @@
       <c r="AB74" t="inlineStr"/>
       <c r="AC74" t="inlineStr"/>
       <c r="AD74" t="inlineStr"/>
-      <c r="AE74" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF74" t="inlineStr"/>
+      <c r="AE74" t="inlineStr"/>
+      <c r="AF74" t="n">
+        <v>0</v>
+      </c>
       <c r="AG74" t="inlineStr"/>
       <c r="AH74" t="inlineStr"/>
+      <c r="AI74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -21980,18 +22059,18 @@
         <v>338</v>
       </c>
       <c r="H75" t="inlineStr"/>
-      <c r="I75" t="n">
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="n">
         <v>10</v>
       </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="n">
-        <v>1</v>
-      </c>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="n">
-        <v>1</v>
-      </c>
-      <c r="N75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="n">
+        <v>1</v>
+      </c>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="n">
+        <v>1</v>
+      </c>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
       <c r="Q75" t="inlineStr"/>
@@ -21999,10 +22078,10 @@
       <c r="S75" t="inlineStr"/>
       <c r="T75" t="inlineStr"/>
       <c r="U75" t="inlineStr"/>
-      <c r="V75" t="n">
-        <v>1</v>
-      </c>
-      <c r="W75" t="inlineStr"/>
+      <c r="V75" t="inlineStr"/>
+      <c r="W75" t="n">
+        <v>1</v>
+      </c>
       <c r="X75" t="inlineStr"/>
       <c r="Y75" t="inlineStr"/>
       <c r="Z75" t="inlineStr"/>
@@ -22010,12 +22089,13 @@
       <c r="AB75" t="inlineStr"/>
       <c r="AC75" t="inlineStr"/>
       <c r="AD75" t="inlineStr"/>
-      <c r="AE75" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF75" t="inlineStr"/>
+      <c r="AE75" t="inlineStr"/>
+      <c r="AF75" t="n">
+        <v>0</v>
+      </c>
       <c r="AG75" t="inlineStr"/>
       <c r="AH75" t="inlineStr"/>
+      <c r="AI75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -22048,23 +22128,23 @@
         <v>186</v>
       </c>
       <c r="H76" t="inlineStr"/>
-      <c r="I76" t="n">
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="n">
         <v>6</v>
       </c>
-      <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
-      <c r="O76" t="n">
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="n">
         <v>2</v>
       </c>
-      <c r="P76" t="inlineStr"/>
       <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="n">
-        <v>1</v>
-      </c>
-      <c r="S76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="n">
+        <v>1</v>
+      </c>
       <c r="T76" t="inlineStr"/>
       <c r="U76" t="inlineStr"/>
       <c r="V76" t="inlineStr"/>
@@ -22076,12 +22156,13 @@
       <c r="AB76" t="inlineStr"/>
       <c r="AC76" t="inlineStr"/>
       <c r="AD76" t="inlineStr"/>
-      <c r="AE76" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF76" t="inlineStr"/>
+      <c r="AE76" t="inlineStr"/>
+      <c r="AF76" t="n">
+        <v>0</v>
+      </c>
       <c r="AG76" t="inlineStr"/>
       <c r="AH76" t="inlineStr"/>
+      <c r="AI76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -22114,20 +22195,20 @@
         <v>157</v>
       </c>
       <c r="H77" t="inlineStr"/>
-      <c r="I77" t="n">
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="n">
         <v>5</v>
       </c>
-      <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr"/>
-      <c r="M77" t="n">
-        <v>1</v>
-      </c>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="n">
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="n">
+        <v>1</v>
+      </c>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="n">
         <v>2</v>
       </c>
-      <c r="P77" t="inlineStr"/>
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr"/>
@@ -22142,12 +22223,13 @@
       <c r="AB77" t="inlineStr"/>
       <c r="AC77" t="inlineStr"/>
       <c r="AD77" t="inlineStr"/>
-      <c r="AE77" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF77" t="inlineStr"/>
+      <c r="AE77" t="inlineStr"/>
+      <c r="AF77" t="n">
+        <v>0</v>
+      </c>
       <c r="AG77" t="inlineStr"/>
       <c r="AH77" t="inlineStr"/>
+      <c r="AI77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -22184,22 +22266,22 @@
           <t>Ignora 1 punto de resistencia a crítico del objetivo al atacar sorprendiendo.</t>
         </is>
       </c>
-      <c r="I78" t="n">
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="n">
         <v>5</v>
       </c>
-      <c r="J78" t="n">
-        <v>1</v>
-      </c>
-      <c r="K78" t="inlineStr"/>
+      <c r="K78" t="n">
+        <v>1</v>
+      </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="n">
-        <v>1</v>
-      </c>
-      <c r="R78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="n">
+        <v>1</v>
+      </c>
       <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr"/>
       <c r="U78" t="inlineStr"/>
@@ -22212,12 +22294,13 @@
       <c r="AB78" t="inlineStr"/>
       <c r="AC78" t="inlineStr"/>
       <c r="AD78" t="inlineStr"/>
-      <c r="AE78" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF78" t="inlineStr"/>
+      <c r="AE78" t="inlineStr"/>
+      <c r="AF78" t="n">
+        <v>0</v>
+      </c>
       <c r="AG78" t="inlineStr"/>
       <c r="AH78" t="inlineStr"/>
+      <c r="AI78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -22254,16 +22337,16 @@
           <t xml:space="preserve">Resistencia a críticos tipo 4, doble resistencia a críticos tipo 2 </t>
         </is>
       </c>
-      <c r="I79" t="n">
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="n">
         <v>4</v>
       </c>
-      <c r="J79" t="n">
+      <c r="K79" t="n">
         <v>2</v>
       </c>
-      <c r="K79" t="n">
-        <v>1</v>
-      </c>
-      <c r="L79" t="inlineStr"/>
+      <c r="L79" t="n">
+        <v>1</v>
+      </c>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
@@ -22282,12 +22365,13 @@
       <c r="AB79" t="inlineStr"/>
       <c r="AC79" t="inlineStr"/>
       <c r="AD79" t="inlineStr"/>
-      <c r="AE79" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF79" t="inlineStr"/>
+      <c r="AE79" t="inlineStr"/>
+      <c r="AF79" t="n">
+        <v>0</v>
+      </c>
       <c r="AG79" t="inlineStr"/>
       <c r="AH79" t="inlineStr"/>
+      <c r="AI79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -22346,16 +22430,17 @@
       <c r="AB80" t="inlineStr"/>
       <c r="AC80" t="inlineStr"/>
       <c r="AD80" t="inlineStr"/>
-      <c r="AE80" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF80" t="inlineStr"/>
-      <c r="AG80" t="inlineStr">
+      <c r="AE80" t="inlineStr"/>
+      <c r="AF80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG80" t="inlineStr"/>
+      <c r="AH80" t="inlineStr">
         <is>
           <t>capcinturon:5</t>
         </is>
       </c>
-      <c r="AH80" t="inlineStr"/>
+      <c r="AI80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -22392,10 +22477,10 @@
           <t>Ranuras para consumibles +3</t>
         </is>
       </c>
-      <c r="I81" t="n">
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="n">
         <v>3</v>
       </c>
-      <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
@@ -22416,16 +22501,17 @@
       <c r="AB81" t="inlineStr"/>
       <c r="AC81" t="inlineStr"/>
       <c r="AD81" t="inlineStr"/>
-      <c r="AE81" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF81" t="inlineStr"/>
-      <c r="AG81" t="inlineStr">
+      <c r="AE81" t="inlineStr"/>
+      <c r="AF81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG81" t="inlineStr"/>
+      <c r="AH81" t="inlineStr">
         <is>
           <t>capcinturon:3</t>
         </is>
       </c>
-      <c r="AH81" t="inlineStr"/>
+      <c r="AI81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -22462,12 +22548,10 @@
           <t>Reduce críticos de cualquier tipo.</t>
         </is>
       </c>
-      <c r="I82" t="n">
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="n">
         <v>10</v>
       </c>
-      <c r="J82" t="n">
-        <v>1</v>
-      </c>
       <c r="K82" t="n">
         <v>1</v>
       </c>
@@ -22480,7 +22564,9 @@
       <c r="N82" t="n">
         <v>1</v>
       </c>
-      <c r="O82" t="inlineStr"/>
+      <c r="O82" t="n">
+        <v>1</v>
+      </c>
       <c r="P82" t="inlineStr"/>
       <c r="Q82" t="inlineStr"/>
       <c r="R82" t="inlineStr"/>
@@ -22496,12 +22582,13 @@
       <c r="AB82" t="inlineStr"/>
       <c r="AC82" t="inlineStr"/>
       <c r="AD82" t="inlineStr"/>
-      <c r="AE82" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF82" t="inlineStr"/>
+      <c r="AE82" t="inlineStr"/>
+      <c r="AF82" t="n">
+        <v>0</v>
+      </c>
       <c r="AG82" t="inlineStr"/>
       <c r="AH82" t="inlineStr"/>
+      <c r="AI82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -22538,10 +22625,10 @@
           <t>Reduce críticos Tipo 2, 4 y 6.</t>
         </is>
       </c>
-      <c r="I83" t="n">
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="n">
         <v>5</v>
       </c>
-      <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr"/>
@@ -22562,12 +22649,13 @@
       <c r="AB83" t="inlineStr"/>
       <c r="AC83" t="inlineStr"/>
       <c r="AD83" t="inlineStr"/>
-      <c r="AE83" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF83" t="inlineStr"/>
+      <c r="AE83" t="inlineStr"/>
+      <c r="AF83" t="n">
+        <v>0</v>
+      </c>
       <c r="AG83" t="inlineStr"/>
       <c r="AH83" t="inlineStr"/>
+      <c r="AI83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -22604,12 +22692,10 @@
           <t>Reduce críticos Tipo 2, 4, 6 y 8.</t>
         </is>
       </c>
-      <c r="I84" t="n">
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="n">
         <v>9</v>
       </c>
-      <c r="J84" t="n">
-        <v>1</v>
-      </c>
       <c r="K84" t="n">
         <v>1</v>
       </c>
@@ -22619,7 +22705,9 @@
       <c r="M84" t="n">
         <v>1</v>
       </c>
-      <c r="N84" t="inlineStr"/>
+      <c r="N84" t="n">
+        <v>1</v>
+      </c>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr"/>
       <c r="Q84" t="inlineStr"/>
@@ -22636,12 +22724,13 @@
       <c r="AB84" t="inlineStr"/>
       <c r="AC84" t="inlineStr"/>
       <c r="AD84" t="inlineStr"/>
-      <c r="AE84" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF84" t="inlineStr"/>
+      <c r="AE84" t="inlineStr"/>
+      <c r="AF84" t="n">
+        <v>0</v>
+      </c>
       <c r="AG84" t="inlineStr"/>
       <c r="AH84" t="inlineStr"/>
+      <c r="AI84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -22678,12 +22767,10 @@
           <t>Reduce críticos Tipo 2, 4, 6 y 8.</t>
         </is>
       </c>
-      <c r="I85" t="n">
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="n">
         <v>9</v>
       </c>
-      <c r="J85" t="n">
-        <v>1</v>
-      </c>
       <c r="K85" t="n">
         <v>1</v>
       </c>
@@ -22693,7 +22780,9 @@
       <c r="M85" t="n">
         <v>1</v>
       </c>
-      <c r="N85" t="inlineStr"/>
+      <c r="N85" t="n">
+        <v>1</v>
+      </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr"/>
       <c r="Q85" t="inlineStr"/>
@@ -22710,12 +22799,13 @@
       <c r="AB85" t="inlineStr"/>
       <c r="AC85" t="inlineStr"/>
       <c r="AD85" t="inlineStr"/>
-      <c r="AE85" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF85" t="inlineStr"/>
+      <c r="AE85" t="inlineStr"/>
+      <c r="AF85" t="n">
+        <v>0</v>
+      </c>
       <c r="AG85" t="inlineStr"/>
       <c r="AH85" t="inlineStr"/>
+      <c r="AI85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -22748,27 +22838,27 @@
         <v>205</v>
       </c>
       <c r="H86" t="inlineStr"/>
-      <c r="I86" t="n">
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="n">
         <v>9</v>
       </c>
-      <c r="J86" t="n">
-        <v>1</v>
-      </c>
-      <c r="K86" t="inlineStr"/>
+      <c r="K86" t="n">
+        <v>1</v>
+      </c>
       <c r="L86" t="inlineStr"/>
-      <c r="M86" t="n">
-        <v>1</v>
-      </c>
-      <c r="N86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="n">
+        <v>1</v>
+      </c>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr"/>
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr"/>
-      <c r="T86" t="n">
-        <v>1</v>
-      </c>
-      <c r="U86" t="inlineStr"/>
+      <c r="T86" t="inlineStr"/>
+      <c r="U86" t="n">
+        <v>1</v>
+      </c>
       <c r="V86" t="inlineStr"/>
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr"/>
@@ -22778,12 +22868,13 @@
       <c r="AB86" t="inlineStr"/>
       <c r="AC86" t="inlineStr"/>
       <c r="AD86" t="inlineStr"/>
-      <c r="AE86" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF86" t="inlineStr"/>
+      <c r="AE86" t="inlineStr"/>
+      <c r="AF86" t="n">
+        <v>0</v>
+      </c>
       <c r="AG86" t="inlineStr"/>
       <c r="AH86" t="inlineStr"/>
+      <c r="AI86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -22820,12 +22911,10 @@
           <t>Reduce críticos Tipo 2, 4, 6 y 8.</t>
         </is>
       </c>
-      <c r="I87" t="n">
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="n">
         <v>6</v>
       </c>
-      <c r="J87" t="n">
-        <v>1</v>
-      </c>
       <c r="K87" t="n">
         <v>1</v>
       </c>
@@ -22835,15 +22924,17 @@
       <c r="M87" t="n">
         <v>1</v>
       </c>
-      <c r="N87" t="inlineStr"/>
+      <c r="N87" t="n">
+        <v>1</v>
+      </c>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr"/>
       <c r="Q87" t="inlineStr"/>
       <c r="R87" t="inlineStr"/>
-      <c r="S87" t="n">
-        <v>1</v>
-      </c>
-      <c r="T87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
+      <c r="T87" t="n">
+        <v>1</v>
+      </c>
       <c r="U87" t="inlineStr"/>
       <c r="V87" t="inlineStr"/>
       <c r="W87" t="inlineStr"/>
@@ -22854,12 +22945,13 @@
       <c r="AB87" t="inlineStr"/>
       <c r="AC87" t="inlineStr"/>
       <c r="AD87" t="inlineStr"/>
-      <c r="AE87" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF87" t="inlineStr"/>
+      <c r="AE87" t="inlineStr"/>
+      <c r="AF87" t="n">
+        <v>0</v>
+      </c>
       <c r="AG87" t="inlineStr"/>
       <c r="AH87" t="inlineStr"/>
+      <c r="AI87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -22896,12 +22988,10 @@
           <t>Reduce críticos Tipo 2, 4, 6, 8 y 10.</t>
         </is>
       </c>
-      <c r="I88" t="n">
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="n">
         <v>8</v>
       </c>
-      <c r="J88" t="n">
-        <v>1</v>
-      </c>
       <c r="K88" t="n">
         <v>1</v>
       </c>
@@ -22914,16 +23004,18 @@
       <c r="N88" t="n">
         <v>1</v>
       </c>
-      <c r="O88" t="inlineStr"/>
+      <c r="O88" t="n">
+        <v>1</v>
+      </c>
       <c r="P88" t="inlineStr"/>
       <c r="Q88" t="inlineStr"/>
       <c r="R88" t="inlineStr"/>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr"/>
-      <c r="U88" t="n">
-        <v>1</v>
-      </c>
-      <c r="V88" t="inlineStr"/>
+      <c r="U88" t="inlineStr"/>
+      <c r="V88" t="n">
+        <v>1</v>
+      </c>
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr"/>
       <c r="Y88" t="inlineStr"/>
@@ -22932,12 +23024,13 @@
       <c r="AB88" t="inlineStr"/>
       <c r="AC88" t="inlineStr"/>
       <c r="AD88" t="inlineStr"/>
-      <c r="AE88" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF88" t="inlineStr"/>
+      <c r="AE88" t="inlineStr"/>
+      <c r="AF88" t="n">
+        <v>0</v>
+      </c>
       <c r="AG88" t="inlineStr"/>
       <c r="AH88" t="inlineStr"/>
+      <c r="AI88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -22974,10 +23067,10 @@
           <t>parry +2</t>
         </is>
       </c>
-      <c r="I89" t="n">
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="n">
         <v>2</v>
       </c>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
@@ -22987,10 +23080,10 @@
       <c r="Q89" t="inlineStr"/>
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="inlineStr"/>
-      <c r="T89" t="n">
+      <c r="T89" t="inlineStr"/>
+      <c r="U89" t="n">
         <v>2</v>
       </c>
-      <c r="U89" t="inlineStr"/>
       <c r="V89" t="inlineStr"/>
       <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr"/>
@@ -23000,12 +23093,13 @@
       <c r="AB89" t="inlineStr"/>
       <c r="AC89" t="inlineStr"/>
       <c r="AD89" t="inlineStr"/>
-      <c r="AE89" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF89" t="inlineStr"/>
+      <c r="AE89" t="inlineStr"/>
+      <c r="AF89" t="n">
+        <v>0</v>
+      </c>
       <c r="AG89" t="inlineStr"/>
       <c r="AH89" t="inlineStr"/>
+      <c r="AI89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -23042,19 +23136,19 @@
           <t>Al curar a un aliado, el portador también recibe 5 HP instantáneos.</t>
         </is>
       </c>
-      <c r="I90" t="n">
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="n">
         <v>4</v>
       </c>
-      <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q90" t="inlineStr"/>
+      <c r="P90" t="inlineStr"/>
+      <c r="Q90" t="n">
+        <v>1</v>
+      </c>
       <c r="R90" t="inlineStr"/>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="inlineStr"/>
@@ -23068,12 +23162,13 @@
       <c r="AB90" t="inlineStr"/>
       <c r="AC90" t="inlineStr"/>
       <c r="AD90" t="inlineStr"/>
-      <c r="AE90" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF90" t="inlineStr"/>
+      <c r="AE90" t="inlineStr"/>
+      <c r="AF90" t="n">
+        <v>0</v>
+      </c>
       <c r="AG90" t="inlineStr"/>
       <c r="AH90" t="inlineStr"/>
+      <c r="AI90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -23110,10 +23205,10 @@
           <t>Dan aspecto de señor fino. No dejan huellas. +1 a todas las tiradas de interacción social</t>
         </is>
       </c>
-      <c r="I91" t="n">
-        <v>1</v>
-      </c>
-      <c r="J91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="n">
+        <v>1</v>
+      </c>
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
@@ -23134,12 +23229,13 @@
       <c r="AB91" t="inlineStr"/>
       <c r="AC91" t="inlineStr"/>
       <c r="AD91" t="inlineStr"/>
-      <c r="AE91" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF91" t="inlineStr"/>
+      <c r="AE91" t="inlineStr"/>
+      <c r="AF91" t="n">
+        <v>0</v>
+      </c>
       <c r="AG91" t="inlineStr"/>
       <c r="AH91" t="inlineStr"/>
+      <c r="AI91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -23176,20 +23272,20 @@
           <t>Reduce críticos Tipo 4, 6 y 8.</t>
         </is>
       </c>
-      <c r="I92" t="n">
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="n">
         <v>6</v>
       </c>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="n">
-        <v>1</v>
-      </c>
+      <c r="K92" t="inlineStr"/>
       <c r="L92" t="n">
         <v>1</v>
       </c>
       <c r="M92" t="n">
         <v>1</v>
       </c>
-      <c r="N92" t="inlineStr"/>
+      <c r="N92" t="n">
+        <v>1</v>
+      </c>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
       <c r="Q92" t="inlineStr"/>
@@ -23206,12 +23302,13 @@
       <c r="AB92" t="inlineStr"/>
       <c r="AC92" t="inlineStr"/>
       <c r="AD92" t="inlineStr"/>
-      <c r="AE92" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF92" t="inlineStr"/>
+      <c r="AE92" t="inlineStr"/>
+      <c r="AF92" t="n">
+        <v>0</v>
+      </c>
       <c r="AG92" t="inlineStr"/>
       <c r="AH92" t="inlineStr"/>
+      <c r="AI92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -23248,21 +23345,21 @@
           <t>Reducción fuerte a críticos tipo 6, leve a 8 y 10</t>
         </is>
       </c>
-      <c r="I93" t="n">
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="n">
         <v>4</v>
       </c>
-      <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
-      <c r="L93" t="n">
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="n">
         <v>2</v>
       </c>
-      <c r="M93" t="n">
-        <v>1</v>
-      </c>
       <c r="N93" t="n">
         <v>1</v>
       </c>
-      <c r="O93" t="inlineStr"/>
+      <c r="O93" t="n">
+        <v>1</v>
+      </c>
       <c r="P93" t="inlineStr"/>
       <c r="Q93" t="inlineStr"/>
       <c r="R93" t="inlineStr"/>
@@ -23278,12 +23375,13 @@
       <c r="AB93" t="inlineStr"/>
       <c r="AC93" t="inlineStr"/>
       <c r="AD93" t="inlineStr"/>
-      <c r="AE93" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF93" t="inlineStr"/>
+      <c r="AE93" t="inlineStr"/>
+      <c r="AF93" t="n">
+        <v>0</v>
+      </c>
       <c r="AG93" t="inlineStr"/>
       <c r="AH93" t="inlineStr"/>
+      <c r="AI93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -23320,24 +23418,24 @@
           <t>inmunidad a armadura rota/arruinada</t>
         </is>
       </c>
-      <c r="I94" t="n">
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="n">
         <v>6</v>
       </c>
-      <c r="J94" t="n">
-        <v>1</v>
-      </c>
-      <c r="K94" t="inlineStr"/>
+      <c r="K94" t="n">
+        <v>1</v>
+      </c>
       <c r="L94" t="inlineStr"/>
-      <c r="M94" t="n">
-        <v>1</v>
-      </c>
-      <c r="N94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="n">
+        <v>1</v>
+      </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr"/>
-      <c r="Q94" t="n">
-        <v>1</v>
-      </c>
-      <c r="R94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="n">
+        <v>1</v>
+      </c>
       <c r="S94" t="inlineStr"/>
       <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr"/>
@@ -23350,12 +23448,13 @@
       <c r="AB94" t="inlineStr"/>
       <c r="AC94" t="inlineStr"/>
       <c r="AD94" t="inlineStr"/>
-      <c r="AE94" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF94" t="inlineStr"/>
+      <c r="AE94" t="inlineStr"/>
+      <c r="AF94" t="n">
+        <v>0</v>
+      </c>
       <c r="AG94" t="inlineStr"/>
       <c r="AH94" t="inlineStr"/>
+      <c r="AI94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -23388,25 +23487,25 @@
         <v>205</v>
       </c>
       <c r="H95" t="inlineStr"/>
-      <c r="I95" t="n">
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="n">
         <v>9</v>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="n">
-        <v>1</v>
-      </c>
+      <c r="K95" t="inlineStr"/>
       <c r="L95" t="n">
         <v>1</v>
       </c>
-      <c r="M95" t="inlineStr"/>
+      <c r="M95" t="n">
+        <v>1</v>
+      </c>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr"/>
       <c r="Q95" t="inlineStr"/>
-      <c r="R95" t="n">
-        <v>1</v>
-      </c>
-      <c r="S95" t="inlineStr"/>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="n">
+        <v>1</v>
+      </c>
       <c r="T95" t="inlineStr"/>
       <c r="U95" t="inlineStr"/>
       <c r="V95" t="inlineStr"/>
@@ -23418,15 +23517,16 @@
       <c r="AB95" t="inlineStr"/>
       <c r="AC95" t="inlineStr"/>
       <c r="AD95" t="inlineStr"/>
-      <c r="AE95" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF95" t="inlineStr"/>
+      <c r="AE95" t="inlineStr"/>
+      <c r="AF95" t="n">
+        <v>0</v>
+      </c>
       <c r="AG95" t="inlineStr"/>
       <c r="AH95" t="inlineStr"/>
+      <c r="AI95" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH95"/>
+  <autoFilter ref="A1:AI95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28386,7 +28486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -28616,12 +28716,12 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Tiene imagen</t>
+          <t>Ocultar en el catálogo</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Solo informativo. Las imágenes NO están en este Excel porque pesan cientos de KB cada una; viven en el programa y se conservan solas al reimportar, siempre que no cambies el ID.</t>
+          <t>(Solo en Defensivos, por ahora.) Con "sí", el ítem no se escribe a ficha.html/vendor-generator.html/gm-tools.html — no aparece para comprar, equipar en creeps, ni en tiendas generadas. Sigue entero en datos/catalogo.json y en este Excel para poder editarlo. Pensado para ítems generados en automático que todavía no se auditaron/balancearon.</t>
         </is>
       </c>
     </row>
@@ -28630,92 +28730,108 @@
       <c r="B25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Tiene imagen</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Solo informativo. Las imágenes NO están en este Excel porque pesan cientos de KB cada una; viven en el programa y se conservan solas al reimportar, siempre que no cambies el ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>CONTENIDO ACTUAL</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Consumibles</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>129 ítems</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Armas</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>85 ítems</t>
-        </is>
-      </c>
+      <c r="B28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Escudos</t>
+          <t>Consumibles</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>23 ítems</t>
+          <t>129 ítems</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Defensivos</t>
+          <t>Armas</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>94 ítems</t>
+          <t>85 ítems</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Accesorios</t>
+          <t>Escudos</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>69 ítems</t>
+          <t>23 ítems</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>Defensivos</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>94 ítems</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Accesorios</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>69 ítems</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
           <t>Otros</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>0 ítems</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>400 ítems</t>
         </is>

</xml_diff>

<commit_message>
Catálogo: 30 ítems de Defensivos ocultos (generados por IA, sin balancear)
El header de la columna nueva tenía un typo ("ocultar del catoolgo") que
no coincidía con ninguna etiqueta conocida, así que leer_excel.py la
trataba como columna desconocida y las 30 marcas "sí" no se leían —
y el aviso correspondiente nunca se veía porque importar.py capturaba
la lista de avisos de leer() pero no la imprimía. Corregido el header a
mano (misma columna, mismos datos) y ahora importar.py imprime los
avisos de lectura, para que un desajuste de columna así no vuelva a
pasar desapercibido.

Con eso: 30 ítems de Defensivos quedan fuera de ficha.html,
vendor-generator.html y gm-tools.html (370 de 400), pero siguen
enteros en datos/catalogo.json y el Excel para auditarlos.
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -17334,7 +17334,11 @@
         <v>93</v>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J6" t="n">
         <v>6</v>
       </c>
@@ -17748,7 +17752,11 @@
           <t>Reduce críticos Tipo 6 y 8.</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J12" t="n">
         <v>6</v>
       </c>
@@ -18247,7 +18255,11 @@
           <t>Reduce críticos tipo 6</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J19" t="n">
         <v>4</v>
       </c>
@@ -18314,7 +18326,11 @@
         <v>111</v>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J20" t="n">
         <v>7</v>
       </c>
@@ -18385,7 +18401,11 @@
           <t>Reduce críticos Tipo 4, 6 y 8. -1 Movimiento.</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J21" t="n">
         <v>6</v>
       </c>
@@ -18456,7 +18476,11 @@
         <v>92</v>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J22" t="n">
         <v>4</v>
       </c>
@@ -18527,7 +18551,11 @@
           <t>Reduce críticos Tipo 2, 6 y 8.</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J23" t="n">
         <v>6</v>
       </c>
@@ -18596,7 +18624,11 @@
         <v>98</v>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J24" t="n">
         <v>6</v>
       </c>
@@ -18937,7 +18969,11 @@
         <v>37</v>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J29" t="n">
         <v>3</v>
       </c>
@@ -19002,7 +19038,11 @@
         <v>41</v>
       </c>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J30" t="n">
         <v>4</v>
       </c>
@@ -19067,7 +19107,11 @@
         <v>38</v>
       </c>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J31" t="n">
         <v>2</v>
       </c>
@@ -19136,7 +19180,11 @@
           <t>Reduce críticos Tipo 6.</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J32" t="n">
         <v>3</v>
       </c>
@@ -19264,7 +19312,11 @@
         <v>32</v>
       </c>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J34" t="n">
         <v>2</v>
       </c>
@@ -19457,7 +19509,11 @@
         <v>42</v>
       </c>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J37" t="n">
         <v>3</v>
       </c>
@@ -19522,7 +19578,11 @@
         <v>37</v>
       </c>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J38" t="n">
         <v>3</v>
       </c>
@@ -19587,7 +19647,11 @@
         <v>37</v>
       </c>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J39" t="n">
         <v>2</v>
       </c>
@@ -19656,7 +19720,11 @@
           <t>Reduce críticos Tipo 8.</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J40" t="n">
         <v>3</v>
       </c>
@@ -19721,7 +19789,11 @@
         <v>56</v>
       </c>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J41" t="n">
         <v>5</v>
       </c>
@@ -19993,7 +20065,11 @@
         <v>42</v>
       </c>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J45" t="n">
         <v>3</v>
       </c>
@@ -20058,7 +20134,11 @@
         <v>46</v>
       </c>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J46" t="n">
         <v>4</v>
       </c>
@@ -20332,7 +20412,11 @@
         <v>34</v>
       </c>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J50" t="n">
         <v>1</v>
       </c>
@@ -20535,7 +20619,11 @@
         <v>34</v>
       </c>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J53" t="n">
         <v>1</v>
       </c>
@@ -21286,7 +21374,11 @@
           <t>+1 a los Bonos máximos, +1 Res.M y +1 Res.CC.</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J64" t="n">
         <v>2</v>
       </c>
@@ -22059,7 +22151,11 @@
         <v>338</v>
       </c>
       <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J75" t="n">
         <v>10</v>
       </c>
@@ -22128,7 +22224,11 @@
         <v>186</v>
       </c>
       <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J76" t="n">
         <v>6</v>
       </c>
@@ -22195,7 +22295,11 @@
         <v>157</v>
       </c>
       <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J77" t="n">
         <v>5</v>
       </c>
@@ -22266,7 +22370,11 @@
           <t>Ignora 1 punto de resistencia a crítico del objetivo al atacar sorprendiendo.</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J78" t="n">
         <v>5</v>
       </c>
@@ -22767,7 +22875,11 @@
           <t>Reduce críticos Tipo 2, 4, 6 y 8.</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J85" t="n">
         <v>9</v>
       </c>
@@ -22838,7 +22950,11 @@
         <v>205</v>
       </c>
       <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J86" t="n">
         <v>9</v>
       </c>
@@ -23487,7 +23603,11 @@
         <v>205</v>
       </c>
       <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
       <c r="J95" t="n">
         <v>9</v>
       </c>
@@ -24128,7 +24248,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Inmunidad a CC (anillo)</t>
+          <t>Inmutabilidad (anillo)</t>
         </is>
       </c>
       <c r="Q8" t="n">
@@ -24136,14 +24256,10 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Inmune a estados de control (Stun, Exhausto, Pajaritos, Cansado): no se le pueden aplicar mientras esté equipado.</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>Inmunidad a CC</t>
-        </is>
-      </c>
+          <t>Mientras esté equipado, se supone inmune a Stun y a Pajaritos. Recordatorio: no hay un preset que cubra exactamente esta combinación — hay que bloquear esos debuffs a mano si se los intentan aplicar.</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
     </row>
@@ -25307,7 +25423,7 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Inmunidad a CC (anillo)</t>
+          <t>Vigor (anillo)</t>
         </is>
       </c>
       <c r="Q25" t="n">
@@ -25315,14 +25431,10 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Inmune a estados de control (Stun, Exhausto, Pajaritos, Cansado): no se le pueden aplicar mientras esté equipado.</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>Inmunidad a CC</t>
-        </is>
-      </c>
+          <t>Mientras esté equipado, se supone inmune a Cansado y Exhausto. Recordatorio: Inmunidad a CC solo cubre Exhausto (Cansado no está tageado como CC) — ese hay que bloqueárselo a mano.</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Catálogo: Sabatones de hueso de troll al día con su Detalle actualizado
El Detalle cambió (ya no menciona Constitución, la Regeneración pasó
de +1 a +5 HP por turno) pero la configuración se había quedado con la
versión vieja: sacado el mod Con +2 y actualizado Regeneración
(sabatones) a +5 HP/turno.
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -31956,9 +31956,7 @@
       <c r="T159" t="inlineStr"/>
       <c r="U159" t="inlineStr"/>
       <c r="V159" t="inlineStr"/>
-      <c r="W159" t="n">
-        <v>2</v>
-      </c>
+      <c r="W159" t="inlineStr"/>
       <c r="X159" t="inlineStr"/>
       <c r="Y159" t="inlineStr"/>
       <c r="Z159" t="inlineStr"/>
@@ -31972,11 +31970,11 @@
         </is>
       </c>
       <c r="AF159" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AG159" t="inlineStr">
         <is>
-          <t>Cura 1 HP cada turno mientras estén equipados.</t>
+          <t>Cura 5 HP cada turno mientras estén equipados.</t>
         </is>
       </c>
       <c r="AH159" t="inlineStr"/>

</xml_diff>

<commit_message>
Catálogo: Sabatones de hueso de troll, ajuste de tipo-crítico invertido
El Detalle volvió a cambiar: ahora Tipo 2 es el que tiene +2 (antes era
Tipo 8), y Tipo 8/4/6 bajan a +1. Ninguno de los dos Excel tenía
todavía este texto guardado — se aplicó igual, tomando la imagen de
referencia del usuario como la versión correcta.
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -31923,7 +31923,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Resistencia a críticos tipo 8: +2. Resistencia a críticos tipos 2, 4 y 6: +1. Movimiento -1. Regeneración +5 HP por turno.</t>
+          <t>Resistencia a críticos tipo 2: +2. Resistencia a críticos tipos 8, 4 y 6: +1. Movimiento -1. Regeneración +5 HP por turno.</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -31935,7 +31935,7 @@
         <v>10</v>
       </c>
       <c r="K159" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L159" t="n">
         <v>1</v>
@@ -31944,7 +31944,7 @@
         <v>1</v>
       </c>
       <c r="N159" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O159" t="inlineStr"/>
       <c r="P159" t="n">

</xml_diff>

<commit_message>
Catálogo: Sabatones de hueso de troll suman Constitución +1
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -31923,7 +31923,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Resistencia a críticos tipo 2: +2. Resistencia a críticos tipos 8, 4 y 6: +1. Movimiento -1. Regeneración +5 HP por turno.</t>
+          <t>Resistencia a críticos tipo 2: +2. Resistencia a críticos tipos 8, 4 y 6: +1. Movimiento -1. Constitución +1. Regeneración +5 HP por turno.</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -31956,7 +31956,9 @@
       <c r="T159" t="inlineStr"/>
       <c r="U159" t="inlineStr"/>
       <c r="V159" t="inlineStr"/>
-      <c r="W159" t="inlineStr"/>
+      <c r="W159" t="n">
+        <v>1</v>
+      </c>
       <c r="X159" t="inlineStr"/>
       <c r="Y159" t="inlineStr"/>
       <c r="Z159" t="inlineStr"/>

</xml_diff>